<commit_message>
Archive original supplier materials with Git LFS
</commit_message>
<xml_diff>
--- a/outputs/机器人本体产品主表.xlsx
+++ b/outputs/机器人本体产品主表.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="决策摘要" sheetId="1" r:id="R06242a5d99524c64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="场景评分" sheetId="2" r:id="Rfab33a3904874aa3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数主表" sheetId="3" r:id="R4144183da65c4d9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题清单" sheetId="4" r:id="Rd5bbee69f4d64883"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源证据" sheetId="5" r:id="Rc0eb9c952cd74709"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="决策摘要" sheetId="1" r:id="R8f89f76bdb56437a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="场景评分" sheetId="2" r:id="R632c708e5fe44dd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数主表" sheetId="3" r:id="Rcbc6f7c0ce194d38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题清单" sheetId="4" r:id="R7d77b1a83b984152"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源证据" sheetId="5" r:id="Re1177449639741f4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -318,7 +318,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EvidenceSources" displayName="EvidenceSources" ref="A3:I14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EvidenceSources" displayName="EvidenceSources" ref="A3:I21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="source_id"/>
     <x:tableColumn id="2" name="model_id"/>
@@ -1475,7 +1475,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re89f68ab153c410c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6200ac30e8d941f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2584,7 +2584,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88ad26e95f4e4255"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d3e26bbeeb0477e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3216,7 +3216,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ff5b907c53843b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ac865f237304d88"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3474,7 +3474,7 @@
         <x:v>D1（擎骏系列）.pdf</x:v>
       </x:c>
       <x:c r="E9" s="15" t="str">
-        <x:v>external-private/智动力/D1（擎骏系列）.pdf</x:v>
+        <x:v>sources/raw/01_智动力/D1（擎骏系列）.pdf</x:v>
       </x:c>
       <x:c r="F9" s="15" t="str"/>
       <x:c r="G9" s="15" t="str">
@@ -3501,7 +3501,7 @@
         <x:v>JUNO2-SD（龙骏系列）.pdf</x:v>
       </x:c>
       <x:c r="E10" s="15" t="str">
-        <x:v>external-private/智动力/JUNO2-SD（龙骏系列）.pdf</x:v>
+        <x:v>sources/raw/01_智动力/JUNO2-SD（龙骏系列）.pdf</x:v>
       </x:c>
       <x:c r="F10" s="15" t="str"/>
       <x:c r="G10" s="15" t="str">
@@ -3528,7 +3528,7 @@
         <x:v>JUNO1-P（智骏系列）.pdf</x:v>
       </x:c>
       <x:c r="E11" s="15" t="str">
-        <x:v>external-private/智动力/JUNO1-P（智骏系列）.pdf</x:v>
+        <x:v>sources/raw/01_智动力/JUNO1-P（智骏系列）.pdf</x:v>
       </x:c>
       <x:c r="F11" s="15" t="str"/>
       <x:c r="G11" s="15" t="str">
@@ -3555,7 +3555,7 @@
         <x:v>L1（灵骏系列）.pdf</x:v>
       </x:c>
       <x:c r="E12" s="15" t="str">
-        <x:v>external-private/智动力/L1（灵骏系列）.pdf</x:v>
+        <x:v>sources/raw/01_智动力/L1（灵骏系列）.pdf</x:v>
       </x:c>
       <x:c r="F12" s="15" t="str"/>
       <x:c r="G12" s="15" t="str">
@@ -3582,7 +3582,7 @@
         <x:v>全尺寸人形机器人Z1开发手册 r26.6.md</x:v>
       </x:c>
       <x:c r="E13" s="15" t="str">
-        <x:v>external-private/智动力/全尺寸人形机器人Z1开发手册 r26.6.md</x:v>
+        <x:v>sources/raw/01_智动力/全尺寸人形机器人Z1开发手册 r26.6.md</x:v>
       </x:c>
       <x:c r="F13" s="15" t="str">
         <x:v>2026-07-25</x:v>
@@ -3599,23 +3599,21 @@
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="15" t="str">
-        <x:v>src_tianji_marvin</x:v>
+        <x:v>src_zdl_ha</x:v>
       </x:c>
       <x:c r="B14" s="15" t="str">
-        <x:v>tianji_marvin_m6ccs</x:v>
+        <x:v>zdl_ha</x:v>
       </x:c>
       <x:c r="C14" s="15" t="str">
         <x:v>供应商PDF</x:v>
       </x:c>
       <x:c r="D14" s="15" t="str">
-        <x:v>Marvin系列 三折页 250721-CN.pdf</x:v>
+        <x:v>人形臂（HA系列）.pdf</x:v>
       </x:c>
       <x:c r="E14" s="15" t="str">
-        <x:v>external-private/天机智能/Marvin系列 三折页 250721-CN.pdf</x:v>
-      </x:c>
-      <x:c r="F14" s="15" t="str">
-        <x:v>2025-07</x:v>
-      </x:c>
+        <x:v>sources/raw/01_智动力/人形臂（HA系列）.pdf</x:v>
+      </x:c>
+      <x:c r="F14" s="15" t="str"/>
       <x:c r="G14" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
@@ -3623,7 +3621,200 @@
         <x:v>中</x:v>
       </x:c>
       <x:c r="I14" s="15" t="str">
+        <x:v>待纳入机械臂专项对比</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="42" customHeight="1">
+      <x:c r="A15" s="15" t="str">
+        <x:v>src_zdl_fa</x:v>
+      </x:c>
+      <x:c r="B15" s="15" t="str">
+        <x:v>zdl_fa</x:v>
+      </x:c>
+      <x:c r="C15" s="15" t="str">
+        <x:v>供应商PDF</x:v>
+      </x:c>
+      <x:c r="D15" s="15" t="str">
+        <x:v>桌面臂（FA系列）.pdf</x:v>
+      </x:c>
+      <x:c r="E15" s="15" t="str">
+        <x:v>sources/raw/01_智动力/桌面臂（FA系列）.pdf</x:v>
+      </x:c>
+      <x:c r="F15" s="15" t="str"/>
+      <x:c r="G15" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H15" s="15" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="I15" s="15" t="str">
+        <x:v>待纳入机械臂专项对比</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="42" customHeight="1">
+      <x:c r="A16" s="15" t="str">
+        <x:v>src_flexiv_rizon4_manual</x:v>
+      </x:c>
+      <x:c r="B16" s="15" t="str">
+        <x:v>flexiv_rizon4</x:v>
+      </x:c>
+      <x:c r="C16" s="15" t="str">
+        <x:v>供应商PDF</x:v>
+      </x:c>
+      <x:c r="D16" s="15" t="str">
+        <x:v>Rizon4 用户手册_V3.0_zh-CN.pdf</x:v>
+      </x:c>
+      <x:c r="E16" s="15" t="str">
+        <x:v>sources/raw/02_非夕_Flexiv/01_Rizon_拂晓/Rizon4 用户手册_V3.0_zh-CN.pdf</x:v>
+      </x:c>
+      <x:c r="F16" s="15" t="str"/>
+      <x:c r="G16" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H16" s="15" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="I16" s="15" t="str">
+        <x:v>待纳入机械臂专项对比</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="42" customHeight="1">
+      <x:c r="A17" s="15" t="str">
+        <x:v>src_flexiv_rizon_datasheet</x:v>
+      </x:c>
+      <x:c r="B17" s="15" t="str">
+        <x:v>flexiv_rizon</x:v>
+      </x:c>
+      <x:c r="C17" s="15" t="str">
+        <x:v>供应商PDF</x:v>
+      </x:c>
+      <x:c r="D17" s="15" t="str">
+        <x:v>拂晓(Rizon)机器人数据表_V2.0_202409.pdf</x:v>
+      </x:c>
+      <x:c r="E17" s="15" t="str">
+        <x:v>sources/raw/02_非夕_Flexiv/01_Rizon_拂晓/拂晓(Rizon)机器人数据表_V2.0_202409.pdf</x:v>
+      </x:c>
+      <x:c r="F17" s="15" t="str">
+        <x:v>2024-09</x:v>
+      </x:c>
+      <x:c r="G17" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H17" s="15" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="I17" s="15" t="str">
+        <x:v>待纳入机械臂专项对比</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="42" customHeight="1">
+      <x:c r="A18" s="15" t="str">
+        <x:v>src_flexiv_grav_manual</x:v>
+      </x:c>
+      <x:c r="B18" s="15" t="str">
+        <x:v>flexiv_grav</x:v>
+      </x:c>
+      <x:c r="C18" s="15" t="str">
+        <x:v>供应商PDF</x:v>
+      </x:c>
+      <x:c r="D18" s="15" t="str">
+        <x:v>星擎用户手册_V1.0_202404(2).pdf</x:v>
+      </x:c>
+      <x:c r="E18" s="15" t="str">
+        <x:v>sources/raw/02_非夕_Flexiv/02_Grav_星擎/星擎用户手册_V1.0_202404(2).pdf</x:v>
+      </x:c>
+      <x:c r="F18" s="15" t="str">
+        <x:v>2024-04</x:v>
+      </x:c>
+      <x:c r="G18" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H18" s="15" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="I18" s="15" t="str">
+        <x:v>末端执行器资料待结构化</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="42" customHeight="1">
+      <x:c r="A19" s="15" t="str">
+        <x:v>src_flexiv_ft_datasheet</x:v>
+      </x:c>
+      <x:c r="B19" s="15" t="str">
+        <x:v>flexiv_ft</x:v>
+      </x:c>
+      <x:c r="C19" s="15" t="str">
+        <x:v>供应商PDF</x:v>
+      </x:c>
+      <x:c r="D19" s="15" t="str">
+        <x:v>拂晓 F_T 传感器数据表_V1.0_zh-CN.pdf</x:v>
+      </x:c>
+      <x:c r="E19" s="15" t="str">
+        <x:v>sources/raw/02_非夕_Flexiv/03_FT_拂晓传感器/拂晓 F_T 传感器数据表_V1.0_zh-CN.pdf</x:v>
+      </x:c>
+      <x:c r="F19" s="15" t="str"/>
+      <x:c r="G19" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H19" s="15" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="I19" s="15" t="str">
+        <x:v>力传感器资料待结构化</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="42" customHeight="1">
+      <x:c r="A20" s="15" t="str">
+        <x:v>src_tianji_marvin</x:v>
+      </x:c>
+      <x:c r="B20" s="15" t="str">
+        <x:v>tianji_marvin_m6ccs</x:v>
+      </x:c>
+      <x:c r="C20" s="15" t="str">
+        <x:v>供应商PDF</x:v>
+      </x:c>
+      <x:c r="D20" s="15" t="str">
+        <x:v>Marvin系列 三折页 250721-CN.pdf</x:v>
+      </x:c>
+      <x:c r="E20" s="15" t="str">
+        <x:v>sources/raw/03_天机智能_Marvin/01_Marvin双臂/Marvin系列 三折页 250721-CN.pdf</x:v>
+      </x:c>
+      <x:c r="F20" s="15" t="str">
+        <x:v>2025-07</x:v>
+      </x:c>
+      <x:c r="G20" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H20" s="15" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="I20" s="15" t="str">
         <x:v>单臂/双臂模块参数，不含标准底盘</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="42" customHeight="1">
+      <x:c r="A21" s="15" t="str">
+        <x:v>src_material_index</x:v>
+      </x:c>
+      <x:c r="B21" s="15" t="str"/>
+      <x:c r="C21" s="15" t="str">
+        <x:v>内部索引</x:v>
+      </x:c>
+      <x:c r="D21" s="15" t="str">
+        <x:v>供应链材料索引.md</x:v>
+      </x:c>
+      <x:c r="E21" s="15" t="str">
+        <x:v>sources/raw/00_索引/供应链材料索引.md</x:v>
+      </x:c>
+      <x:c r="F21" s="15" t="str"/>
+      <x:c r="G21" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H21" s="15" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="I21" s="15" t="str">
+        <x:v>原目录索引的归档副本</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3632,7 +3823,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra76ca5ab740f4230"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re134595142734ffa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Expand humanoid body research and comparison
</commit_message>
<xml_diff>
--- a/outputs/机器人本体产品主表.xlsx
+++ b/outputs/机器人本体产品主表.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="决策摘要" sheetId="1" r:id="R8f89f76bdb56437a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="场景评分" sheetId="2" r:id="R632c708e5fe44dd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数主表" sheetId="3" r:id="Rcbc6f7c0ce194d38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题清单" sheetId="4" r:id="R7d77b1a83b984152"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源证据" sheetId="5" r:id="Re1177449639741f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="决策摘要" sheetId="1" r:id="Rc6adbc6eae404cd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="场景评分" sheetId="2" r:id="Rad89cee4aa3d4cc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数主表" sheetId="3" r:id="R614e916d26b44e97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题清单" sheetId="4" r:id="R448bd1bface44fd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源证据" sheetId="5" r:id="R5f975c33ac3642b0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -234,7 +234,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ScenarioScores" displayName="ScenarioScores" ref="A6:M16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ScenarioScores" displayName="ScenarioScores" ref="A6:M23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="厂商"/>
     <x:tableColumn id="2" name="型号"/>
@@ -255,7 +255,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RobotMasterData" displayName="RobotMasterData" ref="A3:AK13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RobotMasterData" displayName="RobotMasterData" ref="A3:AK20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="37">
     <x:tableColumn id="1" name="model_id"/>
     <x:tableColumn id="2" name="vendor"/>
@@ -300,7 +300,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SupplierQuestions" displayName="SupplierQuestions" ref="A3:J21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SupplierQuestions" displayName="SupplierQuestions" ref="A3:J35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="question_id"/>
     <x:tableColumn id="2" name="vendor"/>
@@ -318,7 +318,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EvidenceSources" displayName="EvidenceSources" ref="A3:I21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EvidenceSources" displayName="EvidenceSources" ref="A3:I35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="source_id"/>
     <x:tableColumn id="2" name="model_id"/>
@@ -656,22 +656,22 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B7" s="15" t="str">
-        <x:v>星尘</x:v>
+        <x:v>星海图</x:v>
       </x:c>
       <x:c r="C7" s="15" t="str">
-        <x:v>Astribot S1</x:v>
+        <x:v>Galaxea R1 Pro 2026</x:v>
       </x:c>
       <x:c r="D7" s="16" t="n">
-        <x:v>3.95</x:v>
+        <x:v>4.1</x:v>
       </x:c>
       <x:c r="E7" s="15" t="str">
-        <x:v>通过待实测</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="F7" s="15" t="str">
         <x:v>条件 POC</x:v>
       </x:c>
       <x:c r="G7" s="15" t="str">
-        <x:v>论文确认全向底盘；量产配置、接口和工业认证资料不足</x:v>
+        <x:v>三舵轮全向和工作空间契合；重复精度0.5mm且机械臂无制动器是主要风险</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="32" customHeight="1">
@@ -679,13 +679,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B8" s="15" t="str">
-        <x:v>智动力</x:v>
+        <x:v>星尘</x:v>
       </x:c>
       <x:c r="C8" s="15" t="str">
-        <x:v>D1 擎骏系列</x:v>
+        <x:v>Astribot S1</x:v>
       </x:c>
       <x:c r="D8" s="16" t="n">
-        <x:v>3.8</x:v>
+        <x:v>3.95</x:v>
       </x:c>
       <x:c r="E8" s="15" t="str">
         <x:v>通过待实测</x:v>
@@ -694,7 +694,7 @@
         <x:v>条件 POC</x:v>
       </x:c>
       <x:c r="G8" s="15" t="str">
-        <x:v>四轮四转明确支持蟹行；整机重且精度和力控证据不足</x:v>
+        <x:v>论文确认全向底盘；量产配置、接口和工业认证资料不足</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="32" customHeight="1">
@@ -702,22 +702,22 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B9" s="15" t="str">
-        <x:v>宇树</x:v>
+        <x:v>Boston Dynamics</x:v>
       </x:c>
       <x:c r="C9" s="15" t="str">
-        <x:v>Unitree G1-D 旗舰版</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="D9" s="16" t="n">
-        <x:v>2.3</x:v>
+        <x:v>3.85</x:v>
       </x:c>
       <x:c r="E9" s="15" t="str">
-        <x:v>不通过</x:v>
+        <x:v>待实测</x:v>
       </x:c>
       <x:c r="F9" s="15" t="str">
-        <x:v>不进入布线 POC</x:v>
+        <x:v>条件 POC</x:v>
       </x:c>
       <x:c r="G9" s="15" t="str">
-        <x:v>差速底盘不能纯横移；更偏数据采集和开发平台</x:v>
+        <x:v>工业可靠性负载和工作空间领先；但双足连续贴线横移、采购与集成开放性待确认</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="32" customHeight="1">
@@ -725,22 +725,22 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B10" s="15" t="str">
-        <x:v>智动力</x:v>
+        <x:v>Figure AI</x:v>
       </x:c>
       <x:c r="C10" s="15" t="str">
-        <x:v>JUNO2-SD 龙骏系列</x:v>
+        <x:v>Figure 03</x:v>
       </x:c>
       <x:c r="D10" s="16" t="n">
-        <x:v>2.15</x:v>
+        <x:v>3.8000000000000003</x:v>
       </x:c>
       <x:c r="E10" s="15" t="str">
-        <x:v>不通过</x:v>
+        <x:v>待实测</x:v>
       </x:c>
       <x:c r="F10" s="15" t="str">
-        <x:v>不进入布线 POC</x:v>
+        <x:v>条件 POC</x:v>
       </x:c>
       <x:c r="G10" s="15" t="str">
-        <x:v>差速底盘为硬伤；重复定位和力控指标未公开</x:v>
+        <x:v>触觉手和量产设计突出；无公开SDK且双足横移节拍与精度未披露</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="32" customHeight="1">
@@ -748,22 +748,22 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B11" s="15" t="str">
-        <x:v>宇树</x:v>
+        <x:v>智动力</x:v>
       </x:c>
       <x:c r="C11" s="15" t="str">
-        <x:v>Unitree G1-D 通用版</x:v>
+        <x:v>D1 擎骏系列</x:v>
       </x:c>
       <x:c r="D11" s="16" t="n">
-        <x:v>2.05</x:v>
+        <x:v>3.8</x:v>
       </x:c>
       <x:c r="E11" s="15" t="str">
-        <x:v>不通过</x:v>
+        <x:v>通过待实测</x:v>
       </x:c>
       <x:c r="F11" s="15" t="str">
-        <x:v>不进入布线 POC</x:v>
+        <x:v>条件 POC</x:v>
       </x:c>
       <x:c r="G11" s="15" t="str">
-        <x:v>官方参数未提供主动移动底盘</x:v>
+        <x:v>四轮四转明确支持蟹行；整机重且精度和力控证据不足</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="32" customHeight="1">
@@ -771,22 +771,22 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B12" s="15" t="str">
-        <x:v>智动力</x:v>
+        <x:v>它石智航</x:v>
       </x:c>
       <x:c r="C12" s="15" t="str">
-        <x:v>JUNO1-P 智骏系列</x:v>
+        <x:v>TARS A1</x:v>
       </x:c>
       <x:c r="D12" s="16" t="n">
-        <x:v>2</x:v>
+        <x:v>3.6500000000000004</x:v>
       </x:c>
       <x:c r="E12" s="15" t="str">
-        <x:v>不通过</x:v>
+        <x:v>待确认</x:v>
       </x:c>
       <x:c r="F12" s="15" t="str">
-        <x:v>不进入布线 POC</x:v>
+        <x:v>条件 POC</x:v>
       </x:c>
       <x:c r="G12" s="15" t="str">
-        <x:v>差速底盘为硬伤；负载和升降能力低于JUNO2</x:v>
+        <x:v>线束任务证据最强；底盘轮型接口参数和规模部署验收数据未公开且内部反馈仍有差距</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="32" customHeight="1">
@@ -794,42 +794,203 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B13" s="15" t="str">
+        <x:v>逐际动力</x:v>
+      </x:c>
+      <x:c r="C13" s="15" t="str">
+        <x:v>LimX Oli EDU</x:v>
+      </x:c>
+      <x:c r="D13" s="16" t="n">
+        <x:v>3.3499999999999996</x:v>
+      </x:c>
+      <x:c r="E13" s="15" t="str">
+        <x:v>待实测</x:v>
+      </x:c>
+      <x:c r="F13" s="15" t="str">
+        <x:v>补齐资料后再评估</x:v>
+      </x:c>
+      <x:c r="G13" s="15" t="str">
+        <x:v>开放开发工具链和全尺寸工作空间较好；双足贴线横移、精度和工业认证需验证</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="32" customHeight="1">
+      <x:c r="A14" s="15" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B14" s="15" t="str">
+        <x:v>逐际动力</x:v>
+      </x:c>
+      <x:c r="C14" s="15" t="str">
+        <x:v>TRON 2 双臂形态</x:v>
+      </x:c>
+      <x:c r="D14" s="16" t="n">
+        <x:v>3.2</x:v>
+      </x:c>
+      <x:c r="E14" s="15" t="str">
+        <x:v>待确认</x:v>
+      </x:c>
+      <x:c r="F14" s="15" t="str">
+        <x:v>补齐资料后再评估</x:v>
+      </x:c>
+      <x:c r="G14" s="15" t="str">
+        <x:v>接口开放且多形态；四向移动是否包含保持朝向纯横移需要供应商确认</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="32" customHeight="1">
+      <x:c r="A15" s="15" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B15" s="15" t="str">
+        <x:v>Tesla</x:v>
+      </x:c>
+      <x:c r="C15" s="15" t="str">
+        <x:v>Optimus</x:v>
+      </x:c>
+      <x:c r="D15" s="16" t="n">
+        <x:v>2.8000000000000003</x:v>
+      </x:c>
+      <x:c r="E15" s="15" t="str">
+        <x:v>待确认</x:v>
+      </x:c>
+      <x:c r="F15" s="15" t="str">
+        <x:v>补齐资料后再评估</x:v>
+      </x:c>
+      <x:c r="G15" s="15" t="str">
+        <x:v>官方工程参数和外部集成方式严重不足；暂不具备正式采购比较条件</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="32" customHeight="1">
+      <x:c r="A16" s="15" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B16" s="15" t="str">
+        <x:v>宇树</x:v>
+      </x:c>
+      <x:c r="C16" s="15" t="str">
+        <x:v>Unitree G1-D 旗舰版</x:v>
+      </x:c>
+      <x:c r="D16" s="16" t="n">
+        <x:v>2.3</x:v>
+      </x:c>
+      <x:c r="E16" s="15" t="str">
+        <x:v>不通过</x:v>
+      </x:c>
+      <x:c r="F16" s="15" t="str">
+        <x:v>不进入布线 POC</x:v>
+      </x:c>
+      <x:c r="G16" s="15" t="str">
+        <x:v>差速底盘不能纯横移；更偏数据采集和开发平台</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="32" customHeight="1">
+      <x:c r="A17" s="15" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B17" s="15" t="str">
         <x:v>智动力</x:v>
       </x:c>
-      <x:c r="C13" s="15" t="str">
+      <x:c r="C17" s="15" t="str">
+        <x:v>JUNO2-SD 龙骏系列</x:v>
+      </x:c>
+      <x:c r="D17" s="16" t="n">
+        <x:v>2.15</x:v>
+      </x:c>
+      <x:c r="E17" s="15" t="str">
+        <x:v>不通过</x:v>
+      </x:c>
+      <x:c r="F17" s="15" t="str">
+        <x:v>不进入布线 POC</x:v>
+      </x:c>
+      <x:c r="G17" s="15" t="str">
+        <x:v>差速底盘为硬伤；重复定位和力控指标未公开</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="32" customHeight="1">
+      <x:c r="A18" s="15" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B18" s="15" t="str">
+        <x:v>宇树</x:v>
+      </x:c>
+      <x:c r="C18" s="15" t="str">
+        <x:v>Unitree G1-D 通用版</x:v>
+      </x:c>
+      <x:c r="D18" s="16" t="n">
+        <x:v>2.05</x:v>
+      </x:c>
+      <x:c r="E18" s="15" t="str">
+        <x:v>不通过</x:v>
+      </x:c>
+      <x:c r="F18" s="15" t="str">
+        <x:v>不进入布线 POC</x:v>
+      </x:c>
+      <x:c r="G18" s="15" t="str">
+        <x:v>官方参数未提供主动移动底盘</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="32" customHeight="1">
+      <x:c r="A19" s="15" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B19" s="15" t="str">
+        <x:v>智动力</x:v>
+      </x:c>
+      <x:c r="C19" s="15" t="str">
+        <x:v>JUNO1-P 智骏系列</x:v>
+      </x:c>
+      <x:c r="D19" s="16" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E19" s="15" t="str">
+        <x:v>不通过</x:v>
+      </x:c>
+      <x:c r="F19" s="15" t="str">
+        <x:v>不进入布线 POC</x:v>
+      </x:c>
+      <x:c r="G19" s="15" t="str">
+        <x:v>差速底盘为硬伤；负载和升降能力低于JUNO2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="32" customHeight="1">
+      <x:c r="A20" s="15" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B20" s="15" t="str">
+        <x:v>智动力</x:v>
+      </x:c>
+      <x:c r="C20" s="15" t="str">
         <x:v>L1 灵骏系列</x:v>
       </x:c>
-      <x:c r="D13" s="16" t="n">
+      <x:c r="D20" s="16" t="n">
         <x:v>1.85</x:v>
       </x:c>
-      <x:c r="E13" s="15" t="str">
+      <x:c r="E20" s="15" t="str">
         <x:v>不通过</x:v>
       </x:c>
-      <x:c r="F13" s="15" t="str">
+      <x:c r="F20" s="15" t="str">
         <x:v>不进入布线 POC</x:v>
       </x:c>
-      <x:c r="G13" s="15" t="str">
+      <x:c r="G20" s="15" t="str">
         <x:v>差速底盘且负载、臂展和躯干能力较弱</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="32" customHeight="1">
-      <x:c r="A15" s="19" t="str">
-        <x:v>说明：综合分不能越过硬门槛。星尘 S1 和智动力 D1 的全向能力仍需实机确认；D1 体积、重量与工程代价较高。</x:v>
-      </x:c>
-      <x:c r="B15" s="19"/>
-      <x:c r="C15" s="19"/>
-      <x:c r="D15" s="19"/>
-      <x:c r="E15" s="19"/>
-      <x:c r="F15" s="19"/>
-      <x:c r="G15" s="19"/>
+    <x:row r="22" ht="32" customHeight="1">
+      <x:c r="A22" s="19" t="str">
+        <x:v>说明：综合分不能越过横移硬门槛和供货资格。双足侧步不等同工业蟹行；Atlas、Figure、Optimus 的采购与SDK开放性需单独判断。</x:v>
+      </x:c>
+      <x:c r="B22" s="19"/>
+      <x:c r="C22" s="19"/>
+      <x:c r="D22" s="19"/>
+      <x:c r="E22" s="19"/>
+      <x:c r="F22" s="19"/>
+      <x:c r="G22" s="19"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A3:G3"/>
-    <x:mergeCell ref="A15:G15"/>
+    <x:mergeCell ref="A22:G22"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="D6:D13">
+  <x:conditionalFormatting sqref="D6:D20">
     <x:cfRule type="colorScale" priority="1">
       <x:colorScale>
         <x:cfvo type="min"/>
@@ -841,7 +1002,7 @@
       </x:colorScale>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="E6:E13">
+  <x:conditionalFormatting sqref="E6:E20">
     <x:cfRule type="cellIs" dxfId="0" priority="2">
       <x:formula>"不通过"</x:formula>
     </x:cfRule>
@@ -1443,11 +1604,312 @@
         <x:v>双臂模块不含标准底盘；集成全向底盘后再评估</x:v>
       </x:c>
     </x:row>
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" s="15" t="str">
+        <x:v>Boston Dynamics</x:v>
+      </x:c>
+      <x:c r="B17" s="15" t="str">
+        <x:v>Atlas</x:v>
+      </x:c>
+      <x:c r="C17" s="15" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="D17" s="15" t="str">
+        <x:v>待实测</x:v>
+      </x:c>
+      <x:c r="E17" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F17" s="15" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G17" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H17" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I17" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J17" s="15" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K17" s="16" t="n">
+        <x:f>IF(C17&lt;&gt;"是","",SUMPRODUCT(E17:J17,$B$4:$G$4))</x:f>
+        <x:v>3.85</x:v>
+      </x:c>
+      <x:c r="L17" s="15" t="str">
+        <x:f>IF(C17&lt;&gt;"是","不参与移动本体排名",IF(D17="不通过","不进入布线POC",IF(K17&gt;=4.2,"优先POC",IF(K17&gt;=3.5,"条件POC","补齐资料后再评估"))))</x:f>
+        <x:v>条件POC</x:v>
+      </x:c>
+      <x:c r="M17" s="15" t="str">
+        <x:v>工业可靠性负载和工作空间领先；但双足连续贴线横移、采购与集成开放性待确认</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="15" t="str">
+        <x:v>Figure AI</x:v>
+      </x:c>
+      <x:c r="B18" s="15" t="str">
+        <x:v>Figure 03</x:v>
+      </x:c>
+      <x:c r="C18" s="15" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="D18" s="15" t="str">
+        <x:v>待实测</x:v>
+      </x:c>
+      <x:c r="E18" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F18" s="15" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G18" s="15" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H18" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I18" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J18" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K18" s="16" t="n">
+        <x:f>IF(C18&lt;&gt;"是","",SUMPRODUCT(E18:J18,$B$4:$G$4))</x:f>
+        <x:v>3.8000000000000003</x:v>
+      </x:c>
+      <x:c r="L18" s="15" t="str">
+        <x:f>IF(C18&lt;&gt;"是","不参与移动本体排名",IF(D18="不通过","不进入布线POC",IF(K18&gt;=4.2,"优先POC",IF(K18&gt;=3.5,"条件POC","补齐资料后再评估"))))</x:f>
+        <x:v>条件POC</x:v>
+      </x:c>
+      <x:c r="M18" s="15" t="str">
+        <x:v>触觉手和量产设计突出；无公开SDK且双足横移节拍与精度未披露</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="15" t="str">
+        <x:v>Tesla</x:v>
+      </x:c>
+      <x:c r="B19" s="15" t="str">
+        <x:v>Optimus</x:v>
+      </x:c>
+      <x:c r="C19" s="15" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="D19" s="15" t="str">
+        <x:v>待确认</x:v>
+      </x:c>
+      <x:c r="E19" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F19" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G19" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H19" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I19" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J19" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K19" s="16" t="n">
+        <x:f>IF(C19&lt;&gt;"是","",SUMPRODUCT(E19:J19,$B$4:$G$4))</x:f>
+        <x:v>2.8000000000000003</x:v>
+      </x:c>
+      <x:c r="L19" s="15" t="str">
+        <x:f>IF(C19&lt;&gt;"是","不参与移动本体排名",IF(D19="不通过","不进入布线POC",IF(K19&gt;=4.2,"优先POC",IF(K19&gt;=3.5,"条件POC","补齐资料后再评估"))))</x:f>
+        <x:v>补齐资料后再评估</x:v>
+      </x:c>
+      <x:c r="M19" s="15" t="str">
+        <x:v>官方工程参数和外部集成方式严重不足；暂不具备正式采购比较条件</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="A20" s="15" t="str">
+        <x:v>逐际动力</x:v>
+      </x:c>
+      <x:c r="B20" s="15" t="str">
+        <x:v>LimX Oli EDU</x:v>
+      </x:c>
+      <x:c r="C20" s="15" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="D20" s="15" t="str">
+        <x:v>待实测</x:v>
+      </x:c>
+      <x:c r="E20" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F20" s="15" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G20" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H20" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I20" s="15" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J20" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K20" s="16" t="n">
+        <x:f>IF(C20&lt;&gt;"是","",SUMPRODUCT(E20:J20,$B$4:$G$4))</x:f>
+        <x:v>3.3499999999999996</x:v>
+      </x:c>
+      <x:c r="L20" s="15" t="str">
+        <x:f>IF(C20&lt;&gt;"是","不参与移动本体排名",IF(D20="不通过","不进入布线POC",IF(K20&gt;=4.2,"优先POC",IF(K20&gt;=3.5,"条件POC","补齐资料后再评估"))))</x:f>
+        <x:v>补齐资料后再评估</x:v>
+      </x:c>
+      <x:c r="M20" s="15" t="str">
+        <x:v>开放开发工具链和全尺寸工作空间较好；双足贴线横移、精度和工业认证需验证</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="30" customHeight="1">
+      <x:c r="A21" s="15" t="str">
+        <x:v>逐际动力</x:v>
+      </x:c>
+      <x:c r="B21" s="15" t="str">
+        <x:v>TRON 2 双臂形态</x:v>
+      </x:c>
+      <x:c r="C21" s="15" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="D21" s="15" t="str">
+        <x:v>待确认</x:v>
+      </x:c>
+      <x:c r="E21" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F21" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G21" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H21" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I21" s="15" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J21" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K21" s="16" t="n">
+        <x:f>IF(C21&lt;&gt;"是","",SUMPRODUCT(E21:J21,$B$4:$G$4))</x:f>
+        <x:v>3.2</x:v>
+      </x:c>
+      <x:c r="L21" s="15" t="str">
+        <x:f>IF(C21&lt;&gt;"是","不参与移动本体排名",IF(D21="不通过","不进入布线POC",IF(K21&gt;=4.2,"优先POC",IF(K21&gt;=3.5,"条件POC","补齐资料后再评估"))))</x:f>
+        <x:v>补齐资料后再评估</x:v>
+      </x:c>
+      <x:c r="M21" s="15" t="str">
+        <x:v>接口开放且多形态；四向移动是否包含保持朝向纯横移需要供应商确认</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="30" customHeight="1">
+      <x:c r="A22" s="15" t="str">
+        <x:v>星海图</x:v>
+      </x:c>
+      <x:c r="B22" s="15" t="str">
+        <x:v>Galaxea R1 Pro 2026</x:v>
+      </x:c>
+      <x:c r="C22" s="15" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="D22" s="15" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="E22" s="15" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F22" s="15" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G22" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H22" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I22" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J22" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K22" s="16" t="n">
+        <x:f>IF(C22&lt;&gt;"是","",SUMPRODUCT(E22:J22,$B$4:$G$4))</x:f>
+        <x:v>4.1</x:v>
+      </x:c>
+      <x:c r="L22" s="15" t="str">
+        <x:f>IF(C22&lt;&gt;"是","不参与移动本体排名",IF(D22="不通过","不进入布线POC",IF(K22&gt;=4.2,"优先POC",IF(K22&gt;=3.5,"条件POC","补齐资料后再评估"))))</x:f>
+        <x:v>条件POC</x:v>
+      </x:c>
+      <x:c r="M22" s="15" t="str">
+        <x:v>三舵轮全向和工作空间契合；重复精度0.5mm且机械臂无制动器是主要风险</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="30" customHeight="1">
+      <x:c r="A23" s="15" t="str">
+        <x:v>它石智航</x:v>
+      </x:c>
+      <x:c r="B23" s="15" t="str">
+        <x:v>TARS A1</x:v>
+      </x:c>
+      <x:c r="C23" s="15" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="D23" s="15" t="str">
+        <x:v>待确认</x:v>
+      </x:c>
+      <x:c r="E23" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F23" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G23" s="15" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H23" s="15" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I23" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J23" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K23" s="16" t="n">
+        <x:f>IF(C23&lt;&gt;"是","",SUMPRODUCT(E23:J23,$B$4:$G$4))</x:f>
+        <x:v>3.6500000000000004</x:v>
+      </x:c>
+      <x:c r="L23" s="15" t="str">
+        <x:f>IF(C23&lt;&gt;"是","不参与移动本体排名",IF(D23="不通过","不进入布线POC",IF(K23&gt;=4.2,"优先POC",IF(K23&gt;=3.5,"条件POC","补齐资料后再评估"))))</x:f>
+        <x:v>条件POC</x:v>
+      </x:c>
+      <x:c r="M23" s="15" t="str">
+        <x:v>线束任务证据最强；底盘轮型接口参数和规模部署验收数据未公开且内部反馈仍有差距</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:M1"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K7:K16">
+  <x:conditionalFormatting sqref="K7:K23">
     <x:cfRule type="colorScale" priority="1">
       <x:colorScale>
         <x:cfvo type="min"/>
@@ -1459,7 +1921,7 @@
       </x:colorScale>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="D7:D16">
+  <x:conditionalFormatting sqref="D7:D23">
     <x:cfRule type="cellIs" dxfId="2" priority="2">
       <x:formula>"不通过"</x:formula>
     </x:cfRule>
@@ -1468,14 +1930,14 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation operator="between" showErrorMessage="1" errorTitle="评分超范围" error="请输入 0 到 5 的整数。" sqref="E7:J16">
+    <x:dataValidation operator="between" showErrorMessage="1" errorTitle="评分超范围" error="请输入 0 到 5 的整数。" sqref="E7:J23">
       <x:formula1>0</x:formula1>
       <x:formula2>5</x:formula2>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6200ac30e8d941f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R728af8975e604a66"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2578,13 +3040,552 @@
         <x:v>单臂参数；不含标准移动底盘，不参加移动本体排名</x:v>
       </x:c>
     </x:row>
+    <x:row r="14" ht="34" customHeight="1">
+      <x:c r="A14" s="15" t="str">
+        <x:v>boston_atlas_2026</x:v>
+      </x:c>
+      <x:c r="B14" s="15" t="str">
+        <x:v>Boston Dynamics</x:v>
+      </x:c>
+      <x:c r="C14" s="15" t="str">
+        <x:v>Atlas</x:v>
+      </x:c>
+      <x:c r="D14" s="15" t="str">
+        <x:v>全尺寸双足工业人形</x:v>
+      </x:c>
+      <x:c r="E14" s="15" t="str">
+        <x:v>早期客户导入</x:v>
+      </x:c>
+      <x:c r="F14" s="15" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="G14" s="15"/>
+      <x:c r="H14" s="15"/>
+      <x:c r="I14" s="15"/>
+      <x:c r="J14" s="15"/>
+      <x:c r="K14" s="15" t="str">
+        <x:v>双足全电驱</x:v>
+      </x:c>
+      <x:c r="L14" s="15" t="str">
+        <x:v>步态可侧移；连续工业横移待验证</x:v>
+      </x:c>
+      <x:c r="M14" s="15"/>
+      <x:c r="N14" s="15" t="n">
+        <x:v>1900</x:v>
+      </x:c>
+      <x:c r="O14" s="15" t="n">
+        <x:v>1900</x:v>
+      </x:c>
+      <x:c r="P14" s="15"/>
+      <x:c r="Q14" s="15"/>
+      <x:c r="R14" s="15" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="S14" s="15"/>
+      <x:c r="T14" s="15"/>
+      <x:c r="U14" s="15"/>
+      <x:c r="V14" s="15"/>
+      <x:c r="W14" s="15" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="X14" s="15" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="Y14" s="15" t="str"/>
+      <x:c r="Z14" s="15"/>
+      <x:c r="AA14" s="15"/>
+      <x:c r="AB14" s="15" t="str">
+        <x:v>触觉感知；全身力控量化指标未公开</x:v>
+      </x:c>
+      <x:c r="AC14" s="15"/>
+      <x:c r="AD14" s="15"/>
+      <x:c r="AE14" s="15" t="str"/>
+      <x:c r="AF14" s="15" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="AG14" s="15" t="str">
+        <x:v>IP67</x:v>
+      </x:c>
+      <x:c r="AH14" s="15" t="str">
+        <x:v>工业任务手/夹具未披露</x:v>
+      </x:c>
+      <x:c r="AI14" s="15" t="str">
+        <x:v>Orbit可对接MES/WMS；支持条码和工作流集成</x:v>
+      </x:c>
+      <x:c r="AJ14" s="15" t="str">
+        <x:v>官方网站</x:v>
+      </x:c>
+      <x:c r="AK14" s="15" t="str">
+        <x:v>全身Reach 2.3m；持续负载30kg/瞬时50kg；自动换电；仅面向选择性早期客户</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="34" customHeight="1">
+      <x:c r="A15" s="15" t="str">
+        <x:v>figure_03</x:v>
+      </x:c>
+      <x:c r="B15" s="15" t="str">
+        <x:v>Figure AI</x:v>
+      </x:c>
+      <x:c r="C15" s="15" t="str">
+        <x:v>Figure 03</x:v>
+      </x:c>
+      <x:c r="D15" s="15" t="str">
+        <x:v>全尺寸双足通用人形</x:v>
+      </x:c>
+      <x:c r="E15" s="15" t="str">
+        <x:v>量产爬坡/客户验证</x:v>
+      </x:c>
+      <x:c r="F15" s="15"/>
+      <x:c r="G15" s="15"/>
+      <x:c r="H15" s="15"/>
+      <x:c r="I15" s="15"/>
+      <x:c r="J15" s="15"/>
+      <x:c r="K15" s="15" t="str">
+        <x:v>双足电驱</x:v>
+      </x:c>
+      <x:c r="L15" s="15" t="str">
+        <x:v>步态可侧移；工业横移精度未披露</x:v>
+      </x:c>
+      <x:c r="M15" s="15" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="N15" s="15" t="n">
+        <x:v>1727</x:v>
+      </x:c>
+      <x:c r="O15" s="15" t="n">
+        <x:v>1727</x:v>
+      </x:c>
+      <x:c r="P15" s="15"/>
+      <x:c r="Q15" s="15"/>
+      <x:c r="R15" s="15" t="n">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="S15" s="15"/>
+      <x:c r="T15" s="15"/>
+      <x:c r="U15" s="15"/>
+      <x:c r="V15" s="15"/>
+      <x:c r="W15" s="15" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="X15" s="15"/>
+      <x:c r="Y15" s="15" t="str"/>
+      <x:c r="Z15" s="15"/>
+      <x:c r="AA15" s="15"/>
+      <x:c r="AB15" s="15" t="str">
+        <x:v>柔顺触觉手；指尖可检测约3g压力</x:v>
+      </x:c>
+      <x:c r="AC15" s="15"/>
+      <x:c r="AD15" s="15"/>
+      <x:c r="AE15" s="15" t="str"/>
+      <x:c r="AF15" s="15" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="AG15" s="15" t="str"/>
+      <x:c r="AH15" s="15" t="str">
+        <x:v>自研触觉灵巧手</x:v>
+      </x:c>
+      <x:c r="AI15" s="15" t="str">
+        <x:v>Helix专有系统；10Gbps毫米波数据卸载；无公开工业SDK</x:v>
+      </x:c>
+      <x:c r="AJ15" s="15" t="str">
+        <x:v>官方网站</x:v>
+      </x:c>
+      <x:c r="AK15" s="15" t="str">
+        <x:v>2.3kWh电池；2kW无线充电；UN38.3；BMW生产验证；接口和采购方式不公开</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="34" customHeight="1">
+      <x:c r="A16" s="15" t="str">
+        <x:v>tesla_optimus</x:v>
+      </x:c>
+      <x:c r="B16" s="15" t="str">
+        <x:v>Tesla</x:v>
+      </x:c>
+      <x:c r="C16" s="15" t="str">
+        <x:v>Optimus</x:v>
+      </x:c>
+      <x:c r="D16" s="15" t="str">
+        <x:v>全尺寸双足通用人形</x:v>
+      </x:c>
+      <x:c r="E16" s="15" t="str">
+        <x:v>产线建设/内部验证</x:v>
+      </x:c>
+      <x:c r="F16" s="15"/>
+      <x:c r="G16" s="15"/>
+      <x:c r="H16" s="15"/>
+      <x:c r="I16" s="15"/>
+      <x:c r="J16" s="15"/>
+      <x:c r="K16" s="15" t="str">
+        <x:v>双足电驱</x:v>
+      </x:c>
+      <x:c r="L16" s="15" t="str">
+        <x:v>工业横移能力与精度未披露</x:v>
+      </x:c>
+      <x:c r="M16" s="15"/>
+      <x:c r="N16" s="15"/>
+      <x:c r="O16" s="15"/>
+      <x:c r="P16" s="15"/>
+      <x:c r="Q16" s="15"/>
+      <x:c r="R16" s="15"/>
+      <x:c r="S16" s="15"/>
+      <x:c r="T16" s="15"/>
+      <x:c r="U16" s="15"/>
+      <x:c r="V16" s="15"/>
+      <x:c r="W16" s="15"/>
+      <x:c r="X16" s="15"/>
+      <x:c r="Y16" s="15" t="str"/>
+      <x:c r="Z16" s="15"/>
+      <x:c r="AA16" s="15"/>
+      <x:c r="AB16" s="15" t="str">
+        <x:v>未公开</x:v>
+      </x:c>
+      <x:c r="AC16" s="15"/>
+      <x:c r="AD16" s="15"/>
+      <x:c r="AE16" s="15" t="str"/>
+      <x:c r="AF16" s="15" t="str"/>
+      <x:c r="AG16" s="15" t="str"/>
+      <x:c r="AH16" s="15" t="str">
+        <x:v>灵巧手</x:v>
+      </x:c>
+      <x:c r="AI16" s="15" t="str">
+        <x:v>专有软硬件栈；未公开第三方SDK</x:v>
+      </x:c>
+      <x:c r="AJ16" s="15" t="str">
+        <x:v>官方网站+投资者披露</x:v>
+      </x:c>
+      <x:c r="AK16" s="15" t="str">
+        <x:v>官方当前页面未披露身高负载续航自由度等可采购规格；不具备供应商选型基线</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="34" customHeight="1">
+      <x:c r="A17" s="15" t="str">
+        <x:v>limx_oli_edu</x:v>
+      </x:c>
+      <x:c r="B17" s="15" t="str">
+        <x:v>逐际动力</x:v>
+      </x:c>
+      <x:c r="C17" s="15" t="str">
+        <x:v>LimX Oli EDU</x:v>
+      </x:c>
+      <x:c r="D17" s="15" t="str">
+        <x:v>全尺寸双足开发平台</x:v>
+      </x:c>
+      <x:c r="E17" s="15" t="str">
+        <x:v>可购/持续迭代</x:v>
+      </x:c>
+      <x:c r="F17" s="15" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="G17" s="15" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H17" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I17" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J17" s="15"/>
+      <x:c r="K17" s="15" t="str">
+        <x:v>双足步行</x:v>
+      </x:c>
+      <x:c r="L17" s="15" t="str">
+        <x:v>步态可侧移；连续贴线横移待实测</x:v>
+      </x:c>
+      <x:c r="M17" s="15" t="n">
+        <x:v>1.389</x:v>
+      </x:c>
+      <x:c r="N17" s="15" t="n">
+        <x:v>1650</x:v>
+      </x:c>
+      <x:c r="O17" s="15" t="n">
+        <x:v>1650</x:v>
+      </x:c>
+      <x:c r="P17" s="15" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="Q17" s="15"/>
+      <x:c r="R17" s="15" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="S17" s="15" t="n">
+        <x:v>700</x:v>
+      </x:c>
+      <x:c r="T17" s="15"/>
+      <x:c r="U17" s="15"/>
+      <x:c r="V17" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="W17" s="15"/>
+      <x:c r="X17" s="15"/>
+      <x:c r="Y17" s="15" t="str"/>
+      <x:c r="Z17" s="15"/>
+      <x:c r="AA17" s="15"/>
+      <x:c r="AB17" s="15" t="str">
+        <x:v>未公开</x:v>
+      </x:c>
+      <x:c r="AC17" s="15"/>
+      <x:c r="AD17" s="15"/>
+      <x:c r="AE17" s="15" t="str">
+        <x:v>RK3588运控+Orin NX 157TOPS感知</x:v>
+      </x:c>
+      <x:c r="AF17" s="15" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AG17" s="15" t="str"/>
+      <x:c r="AH17" s="15" t="str">
+        <x:v>二指夹爪或五指灵巧手</x:v>
+      </x:c>
+      <x:c r="AI17" s="15" t="str">
+        <x:v>WiFi6；蓝牙；USB3；千兆网；Type-C；遥控/传感/底层和上层运动API</x:v>
+      </x:c>
+      <x:c r="AJ17" s="15" t="str">
+        <x:v>官方网站</x:v>
+      </x:c>
+      <x:c r="AK17" s="15" t="str">
+        <x:v>约2h续航；9500mAh抽屉式电池；最大负载3kg；开放度较好但工业精度和认证未公开</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="34" customHeight="1">
+      <x:c r="A18" s="15" t="str">
+        <x:v>limx_tron2_dualarm</x:v>
+      </x:c>
+      <x:c r="B18" s="15" t="str">
+        <x:v>逐际动力</x:v>
+      </x:c>
+      <x:c r="C18" s="15" t="str">
+        <x:v>TRON 2 双臂形态</x:v>
+      </x:c>
+      <x:c r="D18" s="15" t="str">
+        <x:v>多形态双臂移动平台</x:v>
+      </x:c>
+      <x:c r="E18" s="15" t="str">
+        <x:v>可购/持续迭代</x:v>
+      </x:c>
+      <x:c r="F18" s="15"/>
+      <x:c r="G18" s="15" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H18" s="15"/>
+      <x:c r="I18" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J18" s="15"/>
+      <x:c r="K18" s="15" t="str">
+        <x:v>双足/双轮足可换形</x:v>
+      </x:c>
+      <x:c r="L18" s="15" t="str">
+        <x:v>官方称四向移动；纯横移机制待确认</x:v>
+      </x:c>
+      <x:c r="M18" s="15" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N18" s="15"/>
+      <x:c r="O18" s="15"/>
+      <x:c r="P18" s="15"/>
+      <x:c r="Q18" s="15"/>
+      <x:c r="R18" s="15"/>
+      <x:c r="S18" s="15"/>
+      <x:c r="T18" s="15"/>
+      <x:c r="U18" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="V18" s="15" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="W18" s="15"/>
+      <x:c r="X18" s="15"/>
+      <x:c r="Y18" s="15" t="str"/>
+      <x:c r="Z18" s="15" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="AA18" s="15"/>
+      <x:c r="AB18" s="15" t="str">
+        <x:v>双臂安全边界；力控和力传感量化未公开</x:v>
+      </x:c>
+      <x:c r="AC18" s="15"/>
+      <x:c r="AD18" s="15"/>
+      <x:c r="AE18" s="15" t="str">
+        <x:v>Intel Core Ultra拓展模块</x:v>
+      </x:c>
+      <x:c r="AF18" s="15" t="str"/>
+      <x:c r="AG18" s="15" t="str"/>
+      <x:c r="AH18" s="15" t="str">
+        <x:v>夹爪或灵巧手</x:v>
+      </x:c>
+      <x:c r="AI18" s="15" t="str">
+        <x:v>Python；C++；ROS1/ROS2；以太网；USB3；EtherCAT×2；RS485；多电压供电</x:v>
+      </x:c>
+      <x:c r="AJ18" s="15" t="str">
+        <x:v>官方网站</x:v>
+      </x:c>
+      <x:c r="AK18" s="15" t="str">
+        <x:v>双轮足速度3至5m/s；重复定位±0.5mm；遥操延迟100ms；更偏研发和多形态验证</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="34" customHeight="1">
+      <x:c r="A19" s="15" t="str">
+        <x:v>galaxea_r1pro_2026</x:v>
+      </x:c>
+      <x:c r="B19" s="15" t="str">
+        <x:v>星海图</x:v>
+      </x:c>
+      <x:c r="C19" s="15" t="str">
+        <x:v>Galaxea R1 Pro 2026</x:v>
+      </x:c>
+      <x:c r="D19" s="15" t="str">
+        <x:v>轮式双臂仿人形本体</x:v>
+      </x:c>
+      <x:c r="E19" s="15" t="str">
+        <x:v>现货/科研与行业落地</x:v>
+      </x:c>
+      <x:c r="F19" s="15" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="G19" s="15" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H19" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I19" s="15"/>
+      <x:c r="J19" s="15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K19" s="15" t="str">
+        <x:v>三舵轮360度全向底盘</x:v>
+      </x:c>
+      <x:c r="L19" s="15" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="M19" s="15" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="N19" s="15" t="n">
+        <x:v>1700</x:v>
+      </x:c>
+      <x:c r="O19" s="15" t="n">
+        <x:v>1700</x:v>
+      </x:c>
+      <x:c r="P19" s="15" t="n">
+        <x:v>675</x:v>
+      </x:c>
+      <x:c r="Q19" s="15" t="n">
+        <x:v>636</x:v>
+      </x:c>
+      <x:c r="R19" s="15" t="n">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="S19" s="15" t="n">
+        <x:v>620</x:v>
+      </x:c>
+      <x:c r="T19" s="15"/>
+      <x:c r="U19" s="15" t="n">
+        <x:v>3.5</x:v>
+      </x:c>
+      <x:c r="V19" s="15" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="W19" s="15"/>
+      <x:c r="X19" s="15"/>
+      <x:c r="Y19" s="15" t="str"/>
+      <x:c r="Z19" s="15" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="AA19" s="15"/>
+      <x:c r="AB19" s="15" t="str">
+        <x:v>七轴仿人力控机械臂；力传感为选配</x:v>
+      </x:c>
+      <x:c r="AC19" s="15"/>
+      <x:c r="AD19" s="15"/>
+      <x:c r="AE19" s="15" t="str">
+        <x:v>Jetson AGX Orin 32GB 200TOPS</x:v>
+      </x:c>
+      <x:c r="AF19" s="15" t="str"/>
+      <x:c r="AG19" s="15" t="str"/>
+      <x:c r="AH19" s="15" t="str">
+        <x:v>电动平行夹爪</x:v>
+      </x:c>
+      <x:c r="AI19" s="15" t="str">
+        <x:v>USB3；HDMI；千兆以太网；WiFi6；蓝牙</x:v>
+      </x:c>
+      <x:c r="AJ19" s="15" t="str">
+        <x:v>官方产品页+开发文档</x:v>
+      </x:c>
+      <x:c r="AK19" s="15" t="str">
+        <x:v>垂直工作空间0至2m；带夹爪水平半径861mm；夹持力额定150N峰值350N；A2机械臂无制动器需重点评估断电下坠</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="34" customHeight="1">
+      <x:c r="A20" s="15" t="str">
+        <x:v>tars_a1</x:v>
+      </x:c>
+      <x:c r="B20" s="15" t="str">
+        <x:v>它石智航</x:v>
+      </x:c>
+      <x:c r="C20" s="15" t="str">
+        <x:v>TARS A1</x:v>
+      </x:c>
+      <x:c r="D20" s="15" t="str">
+        <x:v>轮式工业具身本体</x:v>
+      </x:c>
+      <x:c r="E20" s="15" t="str">
+        <x:v>产线验证/规模部署计划</x:v>
+      </x:c>
+      <x:c r="F20" s="15"/>
+      <x:c r="G20" s="15"/>
+      <x:c r="H20" s="15"/>
+      <x:c r="I20" s="15"/>
+      <x:c r="J20" s="15"/>
+      <x:c r="K20" s="15" t="str">
+        <x:v>轮式底盘（轮系未公开）</x:v>
+      </x:c>
+      <x:c r="L20" s="15" t="str">
+        <x:v>待确认</x:v>
+      </x:c>
+      <x:c r="M20" s="15"/>
+      <x:c r="N20" s="15"/>
+      <x:c r="O20" s="15"/>
+      <x:c r="P20" s="15"/>
+      <x:c r="Q20" s="15"/>
+      <x:c r="R20" s="15"/>
+      <x:c r="S20" s="15"/>
+      <x:c r="T20" s="15"/>
+      <x:c r="U20" s="15"/>
+      <x:c r="V20" s="15"/>
+      <x:c r="W20" s="15"/>
+      <x:c r="X20" s="15"/>
+      <x:c r="Y20" s="15" t="str"/>
+      <x:c r="Z20" s="15"/>
+      <x:c r="AA20" s="15"/>
+      <x:c r="AB20" s="15" t="str">
+        <x:v>线束亚毫米装配有公开任务证据；本体力控指标未公开</x:v>
+      </x:c>
+      <x:c r="AC20" s="15"/>
+      <x:c r="AD20" s="15"/>
+      <x:c r="AE20" s="15" t="str"/>
+      <x:c r="AF20" s="15" t="str"/>
+      <x:c r="AG20" s="15" t="str"/>
+      <x:c r="AH20" s="15" t="str">
+        <x:v>定制夹爪或DexHand</x:v>
+      </x:c>
+      <x:c r="AI20" s="15" t="str">
+        <x:v>SDK与末端电气接口未公开</x:v>
+      </x:c>
+      <x:c r="AJ20" s="15" t="str">
+        <x:v>客户/政府/吉尼斯+内部沟通</x:v>
+      </x:c>
+      <x:c r="AK20" s="15" t="str">
+        <x:v>公开完成105次每小时亚毫米线束装配纪录；内部沟通显示规模部署验收仍有差距且前期工装耗材投入高</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:AK1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d3e26bbeeb0477e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab0e2da811f447fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3197,11 +4198,403 @@
       <x:c r="I21" s="15" t="str"/>
       <x:c r="J21" s="15" t="str"/>
     </x:row>
+    <x:row r="22" ht="38" customHeight="1">
+      <x:c r="A22" s="15" t="str">
+        <x:v>Q019</x:v>
+      </x:c>
+      <x:c r="B22" s="15" t="str">
+        <x:v>Boston Dynamics</x:v>
+      </x:c>
+      <x:c r="C22" s="15" t="str">
+        <x:v>Atlas</x:v>
+      </x:c>
+      <x:c r="D22" s="15" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E22" s="15" t="str">
+        <x:v>底盘/步态</x:v>
+      </x:c>
+      <x:c r="F22" s="15" t="str">
+        <x:v>能否保持上身朝向工装完成连续2米横移并给出轨迹与末端误差</x:v>
+      </x:c>
+      <x:c r="G22" s="15" t="str">
+        <x:v>官网仅说明动态双足能力</x:v>
+      </x:c>
+      <x:c r="H22" s="15" t="str">
+        <x:v>待供应商回复</x:v>
+      </x:c>
+      <x:c r="I22" s="15" t="str"/>
+      <x:c r="J22" s="15" t="str"/>
+    </x:row>
+    <x:row r="23" ht="38" customHeight="1">
+      <x:c r="A23" s="15" t="str">
+        <x:v>Q020</x:v>
+      </x:c>
+      <x:c r="B23" s="15" t="str">
+        <x:v>Boston Dynamics</x:v>
+      </x:c>
+      <x:c r="C23" s="15" t="str">
+        <x:v>Atlas</x:v>
+      </x:c>
+      <x:c r="D23" s="15" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="E23" s="15" t="str">
+        <x:v>采购与集成</x:v>
+      </x:c>
+      <x:c r="F23" s="15" t="str">
+        <x:v>中国工厂能否采购并开放任务开发、末端工具和MES接口</x:v>
+      </x:c>
+      <x:c r="G23" s="15" t="str">
+        <x:v>当前仅面向选择性早期客户且Orbit为专有平台</x:v>
+      </x:c>
+      <x:c r="H23" s="15" t="str">
+        <x:v>待供应商回复</x:v>
+      </x:c>
+      <x:c r="I23" s="15" t="str"/>
+      <x:c r="J23" s="15" t="str"/>
+    </x:row>
+    <x:row r="24" ht="38" customHeight="1">
+      <x:c r="A24" s="15" t="str">
+        <x:v>Q021</x:v>
+      </x:c>
+      <x:c r="B24" s="15" t="str">
+        <x:v>Figure AI</x:v>
+      </x:c>
+      <x:c r="C24" s="15" t="str">
+        <x:v>Figure 03</x:v>
+      </x:c>
+      <x:c r="D24" s="15" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E24" s="15" t="str">
+        <x:v>步态与精度</x:v>
+      </x:c>
+      <x:c r="F24" s="15" t="str">
+        <x:v>侧移后双手TCP重定位误差、停稳时间和连续运行节拍是多少</x:v>
+      </x:c>
+      <x:c r="G24" s="15" t="str">
+        <x:v>官网未披露工业步态精度</x:v>
+      </x:c>
+      <x:c r="H24" s="15" t="str">
+        <x:v>待供应商回复</x:v>
+      </x:c>
+      <x:c r="I24" s="15" t="str"/>
+      <x:c r="J24" s="15" t="str"/>
+    </x:row>
+    <x:row r="25" ht="38" customHeight="1">
+      <x:c r="A25" s="15" t="str">
+        <x:v>Q022</x:v>
+      </x:c>
+      <x:c r="B25" s="15" t="str">
+        <x:v>Figure AI</x:v>
+      </x:c>
+      <x:c r="C25" s="15" t="str">
+        <x:v>Figure 03</x:v>
+      </x:c>
+      <x:c r="D25" s="15" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E25" s="15" t="str">
+        <x:v>接口</x:v>
+      </x:c>
+      <x:c r="F25" s="15" t="str">
+        <x:v>是否提供第三方SDK、末端机械接口、电气接口和离线部署能力</x:v>
+      </x:c>
+      <x:c r="G25" s="15" t="str">
+        <x:v>公开资料仅描述Helix专有系统</x:v>
+      </x:c>
+      <x:c r="H25" s="15" t="str">
+        <x:v>待供应商回复</x:v>
+      </x:c>
+      <x:c r="I25" s="15" t="str"/>
+      <x:c r="J25" s="15" t="str"/>
+    </x:row>
+    <x:row r="26" ht="38" customHeight="1">
+      <x:c r="A26" s="15" t="str">
+        <x:v>Q023</x:v>
+      </x:c>
+      <x:c r="B26" s="15" t="str">
+        <x:v>Tesla</x:v>
+      </x:c>
+      <x:c r="C26" s="15" t="str">
+        <x:v>Optimus</x:v>
+      </x:c>
+      <x:c r="D26" s="15" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E26" s="15" t="str">
+        <x:v>可采购性</x:v>
+      </x:c>
+      <x:c r="F26" s="15" t="str">
+        <x:v>是否提供外部销售、工程规格书、SDK和售后服务边界</x:v>
+      </x:c>
+      <x:c r="G26" s="15" t="str">
+        <x:v>官方尚未给出采购规格</x:v>
+      </x:c>
+      <x:c r="H26" s="15" t="str">
+        <x:v>待供应商回复</x:v>
+      </x:c>
+      <x:c r="I26" s="15" t="str"/>
+      <x:c r="J26" s="15" t="str"/>
+    </x:row>
+    <x:row r="27" ht="38" customHeight="1">
+      <x:c r="A27" s="15" t="str">
+        <x:v>Q024</x:v>
+      </x:c>
+      <x:c r="B27" s="15" t="str">
+        <x:v>逐际动力</x:v>
+      </x:c>
+      <x:c r="C27" s="15" t="str">
+        <x:v>LimX Oli EDU</x:v>
+      </x:c>
+      <x:c r="D27" s="15" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E27" s="15" t="str">
+        <x:v>横移POC</x:v>
+      </x:c>
+      <x:c r="F27" s="15" t="str">
+        <x:v>能否在保持胸部朝向的情况下完成连续贴线横移并量化足端稳定和末端误差</x:v>
+      </x:c>
+      <x:c r="G27" s="15" t="str">
+        <x:v>官网只披露行走速度</x:v>
+      </x:c>
+      <x:c r="H27" s="15" t="str">
+        <x:v>待POC</x:v>
+      </x:c>
+      <x:c r="I27" s="15" t="str"/>
+      <x:c r="J27" s="15" t="str"/>
+    </x:row>
+    <x:row r="28" ht="38" customHeight="1">
+      <x:c r="A28" s="15" t="str">
+        <x:v>Q025</x:v>
+      </x:c>
+      <x:c r="B28" s="15" t="str">
+        <x:v>逐际动力</x:v>
+      </x:c>
+      <x:c r="C28" s="15" t="str">
+        <x:v>LimX Oli EDU</x:v>
+      </x:c>
+      <x:c r="D28" s="15" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="E28" s="15" t="str">
+        <x:v>工业可靠性</x:v>
+      </x:c>
+      <x:c r="F28" s="15" t="str">
+        <x:v>重复定位精度、IP等级、MTBF、连续运行和电池循环寿命是多少</x:v>
+      </x:c>
+      <x:c r="G28" s="15" t="str">
+        <x:v>公开资料未披露</x:v>
+      </x:c>
+      <x:c r="H28" s="15" t="str">
+        <x:v>待供应商回复</x:v>
+      </x:c>
+      <x:c r="I28" s="15" t="str"/>
+      <x:c r="J28" s="15" t="str"/>
+    </x:row>
+    <x:row r="29" ht="38" customHeight="1">
+      <x:c r="A29" s="15" t="str">
+        <x:v>Q026</x:v>
+      </x:c>
+      <x:c r="B29" s="15" t="str">
+        <x:v>逐际动力</x:v>
+      </x:c>
+      <x:c r="C29" s="15" t="str">
+        <x:v>TRON 2 双臂形态</x:v>
+      </x:c>
+      <x:c r="D29" s="15" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E29" s="15" t="str">
+        <x:v>底盘</x:v>
+      </x:c>
+      <x:c r="F29" s="15" t="str">
+        <x:v>官方四向移动是否包含无需转向的纯横移；双轮足转向结构是什么</x:v>
+      </x:c>
+      <x:c r="G29" s="15" t="str">
+        <x:v>官网表述不足以判断蟹行能力</x:v>
+      </x:c>
+      <x:c r="H29" s="15" t="str">
+        <x:v>待供应商回复</x:v>
+      </x:c>
+      <x:c r="I29" s="15" t="str"/>
+      <x:c r="J29" s="15" t="str"/>
+    </x:row>
+    <x:row r="30" ht="38" customHeight="1">
+      <x:c r="A30" s="15" t="str">
+        <x:v>Q027</x:v>
+      </x:c>
+      <x:c r="B30" s="15" t="str">
+        <x:v>逐际动力</x:v>
+      </x:c>
+      <x:c r="C30" s="15" t="str">
+        <x:v>TRON 2 双臂形态</x:v>
+      </x:c>
+      <x:c r="D30" s="15" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="E30" s="15" t="str">
+        <x:v>力控</x:v>
+      </x:c>
+      <x:c r="F30" s="15" t="str">
+        <x:v>双臂是否具有关节力矩或末端六维力传感；控制频率和量化精度是多少</x:v>
+      </x:c>
+      <x:c r="G30" s="15" t="str">
+        <x:v>只公开安全边界未公开力控参数</x:v>
+      </x:c>
+      <x:c r="H30" s="15" t="str">
+        <x:v>待供应商回复</x:v>
+      </x:c>
+      <x:c r="I30" s="15" t="str"/>
+      <x:c r="J30" s="15" t="str"/>
+    </x:row>
+    <x:row r="31" ht="38" customHeight="1">
+      <x:c r="A31" s="15" t="str">
+        <x:v>Q028</x:v>
+      </x:c>
+      <x:c r="B31" s="15" t="str">
+        <x:v>星海图</x:v>
+      </x:c>
+      <x:c r="C31" s="15" t="str">
+        <x:v>R1 Pro 2026</x:v>
+      </x:c>
+      <x:c r="D31" s="15" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E31" s="15" t="str">
+        <x:v>断电安全</x:v>
+      </x:c>
+      <x:c r="F31" s="15" t="str">
+        <x:v>A2机械臂无制动器时如何防止断电下坠、夹具碰撞和线束损伤</x:v>
+      </x:c>
+      <x:c r="G31" s="15" t="str">
+        <x:v>官方开发文档明确无制动器</x:v>
+      </x:c>
+      <x:c r="H31" s="15" t="str">
+        <x:v>待供应商回复</x:v>
+      </x:c>
+      <x:c r="I31" s="15" t="str"/>
+      <x:c r="J31" s="15" t="str"/>
+    </x:row>
+    <x:row r="32" ht="38" customHeight="1">
+      <x:c r="A32" s="15" t="str">
+        <x:v>Q029</x:v>
+      </x:c>
+      <x:c r="B32" s="15" t="str">
+        <x:v>星海图</x:v>
+      </x:c>
+      <x:c r="C32" s="15" t="str">
+        <x:v>R1 Pro 2026</x:v>
+      </x:c>
+      <x:c r="D32" s="15" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E32" s="15" t="str">
+        <x:v>整链路精度</x:v>
+      </x:c>
+      <x:c r="F32" s="15" t="str">
+        <x:v>横移停稳后视觉重定位与双手TCP误差是多少；能否稳定插接端子</x:v>
+      </x:c>
+      <x:c r="G32" s="15" t="str">
+        <x:v>机械臂重复定位精度为0.5mm</x:v>
+      </x:c>
+      <x:c r="H32" s="15" t="str">
+        <x:v>待POC</x:v>
+      </x:c>
+      <x:c r="I32" s="15" t="str"/>
+      <x:c r="J32" s="15" t="str"/>
+    </x:row>
+    <x:row r="33" ht="38" customHeight="1">
+      <x:c r="A33" s="15" t="str">
+        <x:v>Q030</x:v>
+      </x:c>
+      <x:c r="B33" s="15" t="str">
+        <x:v>它石智航</x:v>
+      </x:c>
+      <x:c r="C33" s="15" t="str">
+        <x:v>TARS A1</x:v>
+      </x:c>
+      <x:c r="D33" s="15" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E33" s="15" t="str">
+        <x:v>本体参数</x:v>
+      </x:c>
+      <x:c r="F33" s="15" t="str">
+        <x:v>底盘轮型、是否支持纯横移、臂展、负载、自由度、续航和IP等级是什么</x:v>
+      </x:c>
+      <x:c r="G33" s="15" t="str">
+        <x:v>公开任务成果多但本体规格缺失</x:v>
+      </x:c>
+      <x:c r="H33" s="15" t="str">
+        <x:v>待供应商回复</x:v>
+      </x:c>
+      <x:c r="I33" s="15" t="str"/>
+      <x:c r="J33" s="15" t="str"/>
+    </x:row>
+    <x:row r="34" ht="38" customHeight="1">
+      <x:c r="A34" s="15" t="str">
+        <x:v>Q031</x:v>
+      </x:c>
+      <x:c r="B34" s="15" t="str">
+        <x:v>它石智航</x:v>
+      </x:c>
+      <x:c r="C34" s="15" t="str">
+        <x:v>TARS A1</x:v>
+      </x:c>
+      <x:c r="D34" s="15" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E34" s="15" t="str">
+        <x:v>规模验收</x:v>
+      </x:c>
+      <x:c r="F34" s="15" t="str">
+        <x:v>已部署机器人按工序的节拍、一次成功率、OEE、损伤率、人工介入率和最终验收比例是多少</x:v>
+      </x:c>
+      <x:c r="G34" s="15" t="str">
+        <x:v>内部沟通反馈百台部署要求尚未达标</x:v>
+      </x:c>
+      <x:c r="H34" s="15" t="str">
+        <x:v>待供应商回复</x:v>
+      </x:c>
+      <x:c r="I34" s="15" t="str"/>
+      <x:c r="J34" s="15" t="str"/>
+    </x:row>
+    <x:row r="35" ht="38" customHeight="1">
+      <x:c r="A35" s="15" t="str">
+        <x:v>Q032</x:v>
+      </x:c>
+      <x:c r="B35" s="15" t="str">
+        <x:v>它石智航</x:v>
+      </x:c>
+      <x:c r="C35" s="15" t="str">
+        <x:v>TARS A1</x:v>
+      </x:c>
+      <x:c r="D35" s="15" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E35" s="15" t="str">
+        <x:v>项目经济性</x:v>
+      </x:c>
+      <x:c r="F35" s="15" t="str">
+        <x:v>按2.5年回本目标给出本体、场地、工装板、接插件耗材、夹爪迭代、MES集成和维护全成本</x:v>
+      </x:c>
+      <x:c r="G35" s="15" t="str">
+        <x:v>前期场地工装和端子损耗可能显著</x:v>
+      </x:c>
+      <x:c r="H35" s="15" t="str">
+        <x:v>待供应商回复</x:v>
+      </x:c>
+      <x:c r="I35" s="15" t="str"/>
+      <x:c r="J35" s="15" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J1"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="D4:D21">
+  <x:conditionalFormatting sqref="D4:D35">
     <x:cfRule type="cellIs" dxfId="4" priority="1">
       <x:formula>"P0"</x:formula>
     </x:cfRule>
@@ -3210,13 +4603,13 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="H4:H21">
+    <x:dataValidation type="list" sqref="H4:H35">
       <x:formula1>"待供应商回复,待POC,待IT联调,进行中,已关闭,不适用"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ac865f237304d88"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01a047f617b34a1b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3817,13 +5210,403 @@
         <x:v>原目录索引的归档副本</x:v>
       </x:c>
     </x:row>
+    <x:row r="22" ht="42" customHeight="1">
+      <x:c r="A22" s="15" t="str">
+        <x:v>src_boston_atlas</x:v>
+      </x:c>
+      <x:c r="B22" s="15" t="str">
+        <x:v>boston_atlas_2026</x:v>
+      </x:c>
+      <x:c r="C22" s="15" t="str">
+        <x:v>官方网站</x:v>
+      </x:c>
+      <x:c r="D22" s="15" t="str">
+        <x:v>Atlas产品与规格</x:v>
+      </x:c>
+      <x:c r="E22" s="15" t="str">
+        <x:v>https://bostondynamics.com/products/atlas/</x:v>
+      </x:c>
+      <x:c r="F22" s="15" t="str"/>
+      <x:c r="G22" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H22" s="15" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="I22" s="15" t="str">
+        <x:v>披露56自由度、负载、续航、IP67、工作范围和Orbit集成</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="42" customHeight="1">
+      <x:c r="A23" s="15" t="str">
+        <x:v>src_figure03_product</x:v>
+      </x:c>
+      <x:c r="B23" s="15" t="str">
+        <x:v>figure_03</x:v>
+      </x:c>
+      <x:c r="C23" s="15" t="str">
+        <x:v>官方网站</x:v>
+      </x:c>
+      <x:c r="D23" s="15" t="str">
+        <x:v>Figure 03产品页</x:v>
+      </x:c>
+      <x:c r="E23" s="15" t="str">
+        <x:v>https://www.figure.ai/figure</x:v>
+      </x:c>
+      <x:c r="F23" s="15" t="str"/>
+      <x:c r="G23" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H23" s="15" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="I23" s="15" t="str">
+        <x:v>披露身高、重量、负载、速度和续航</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="42" customHeight="1">
+      <x:c r="A24" s="15" t="str">
+        <x:v>src_figure03_intro</x:v>
+      </x:c>
+      <x:c r="B24" s="15" t="str">
+        <x:v>figure_03</x:v>
+      </x:c>
+      <x:c r="C24" s="15" t="str">
+        <x:v>官方技术文章</x:v>
+      </x:c>
+      <x:c r="D24" s="15" t="str">
+        <x:v>Introducing Figure 03</x:v>
+      </x:c>
+      <x:c r="E24" s="15" t="str">
+        <x:v>https://www.figure.ai/news/introducing-figure-03</x:v>
+      </x:c>
+      <x:c r="F24" s="15" t="str">
+        <x:v>2025-10-09</x:v>
+      </x:c>
+      <x:c r="G24" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H24" s="15" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="I24" s="15" t="str">
+        <x:v>披露触觉、感知、充电、电池安全和量产设计</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="42" customHeight="1">
+      <x:c r="A25" s="15" t="str">
+        <x:v>src_figure03_bmw</x:v>
+      </x:c>
+      <x:c r="B25" s="15" t="str">
+        <x:v>figure_03</x:v>
+      </x:c>
+      <x:c r="C25" s="15" t="str">
+        <x:v>官方客户进展</x:v>
+      </x:c>
+      <x:c r="D25" s="15" t="str">
+        <x:v>F.03 Arrives at BMW</x:v>
+      </x:c>
+      <x:c r="E25" s="15" t="str">
+        <x:v>https://www.figure.ai/news/f-03-at-bmw</x:v>
+      </x:c>
+      <x:c r="F25" s="15" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="G25" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H25" s="15" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="I25" s="15" t="str">
+        <x:v>披露BMW工厂物流验证和全身操作</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="42" customHeight="1">
+      <x:c r="A26" s="15" t="str">
+        <x:v>src_tesla_ai</x:v>
+      </x:c>
+      <x:c r="B26" s="15" t="str">
+        <x:v>tesla_optimus</x:v>
+      </x:c>
+      <x:c r="C26" s="15" t="str">
+        <x:v>官方网站</x:v>
+      </x:c>
+      <x:c r="D26" s="15" t="str">
+        <x:v>Tesla AI and Robotics</x:v>
+      </x:c>
+      <x:c r="E26" s="15" t="str">
+        <x:v>https://www.tesla.com/AI</x:v>
+      </x:c>
+      <x:c r="F26" s="15" t="str"/>
+      <x:c r="G26" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H26" s="15" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="I26" s="15" t="str">
+        <x:v>仅说明双足通用自主机器人目标；未给工程规格</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="42" customHeight="1">
+      <x:c r="A27" s="15" t="str">
+        <x:v>src_tesla_2026q2</x:v>
+      </x:c>
+      <x:c r="B27" s="15" t="str">
+        <x:v>tesla_optimus</x:v>
+      </x:c>
+      <x:c r="C27" s="15" t="str">
+        <x:v>官方投资者文件</x:v>
+      </x:c>
+      <x:c r="D27" s="15" t="str">
+        <x:v>Tesla 2026 Q2 Update</x:v>
+      </x:c>
+      <x:c r="E27" s="15" t="str">
+        <x:v>https://ir.tesla.com/_flysystem/s3/sec/000162828026049213/tsla-20260722-gen.pdf</x:v>
+      </x:c>
+      <x:c r="F27" s="15" t="str">
+        <x:v>2026-07-22</x:v>
+      </x:c>
+      <x:c r="G27" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H27" s="15" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="I27" s="15" t="str">
+        <x:v>披露Optimus产线建设与训练数据用途；未给本体规格</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="42" customHeight="1">
+      <x:c r="A28" s="15" t="str">
+        <x:v>src_limx_oli</x:v>
+      </x:c>
+      <x:c r="B28" s="15" t="str">
+        <x:v>limx_oli_edu</x:v>
+      </x:c>
+      <x:c r="C28" s="15" t="str">
+        <x:v>官方网站</x:v>
+      </x:c>
+      <x:c r="D28" s="15" t="str">
+        <x:v>LimX Oli产品参数</x:v>
+      </x:c>
+      <x:c r="E28" s="15" t="str">
+        <x:v>https://www.limxdynamics.com/zh/products/oli/spec</x:v>
+      </x:c>
+      <x:c r="F28" s="15" t="str"/>
+      <x:c r="G28" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H28" s="15" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="I28" s="15" t="str">
+        <x:v>披露自由度、尺寸、负载、续航、算力和开发接口</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="42" customHeight="1">
+      <x:c r="A29" s="15" t="str">
+        <x:v>src_limx_tron2</x:v>
+      </x:c>
+      <x:c r="B29" s="15" t="str">
+        <x:v>limx_tron2_dualarm</x:v>
+      </x:c>
+      <x:c r="C29" s="15" t="str">
+        <x:v>官方网站</x:v>
+      </x:c>
+      <x:c r="D29" s="15" t="str">
+        <x:v>TRON 2产品参数</x:v>
+      </x:c>
+      <x:c r="E29" s="15" t="str">
+        <x:v>https://www.limxdynamics.com/zh/products/tron2/spec</x:v>
+      </x:c>
+      <x:c r="F29" s="15" t="str"/>
+      <x:c r="G29" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H29" s="15" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="I29" s="15" t="str">
+        <x:v>披露双臂负载精度、多形态移动、接口和开发工具</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="42" customHeight="1">
+      <x:c r="A30" s="15" t="str">
+        <x:v>src_galaxea_r1pro_product</x:v>
+      </x:c>
+      <x:c r="B30" s="15" t="str">
+        <x:v>galaxea_r1pro_2026</x:v>
+      </x:c>
+      <x:c r="C30" s="15" t="str">
+        <x:v>官方网站</x:v>
+      </x:c>
+      <x:c r="D30" s="15" t="str">
+        <x:v>R1 Pro产品参数</x:v>
+      </x:c>
+      <x:c r="E30" s="15" t="str">
+        <x:v>https://galaxea-ai.com/cn/products/R1-Pro</x:v>
+      </x:c>
+      <x:c r="F30" s="15" t="str"/>
+      <x:c r="G30" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H30" s="15" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="I30" s="15" t="str">
+        <x:v>披露三舵轮全向底盘、双臂负载、工作空间和算力</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="42" customHeight="1">
+      <x:c r="A31" s="15" t="str">
+        <x:v>src_galaxea_r1pro_docs</x:v>
+      </x:c>
+      <x:c r="B31" s="15" t="str">
+        <x:v>galaxea_r1pro_2026</x:v>
+      </x:c>
+      <x:c r="C31" s="15" t="str">
+        <x:v>官方开发文档</x:v>
+      </x:c>
+      <x:c r="D31" s="15" t="str">
+        <x:v>R1 Pro 2026硬件说明</x:v>
+      </x:c>
+      <x:c r="E31" s="15" t="str">
+        <x:v>https://docs.galaxea-dynamics.com/R1Pro/docs/2026/</x:v>
+      </x:c>
+      <x:c r="F31" s="15" t="str"/>
+      <x:c r="G31" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H31" s="15" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="I31" s="15" t="str">
+        <x:v>披露重量、电池、夹爪、接口和机械臂无制动器风险</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="42" customHeight="1">
+      <x:c r="A32" s="15" t="str">
+        <x:v>src_tars_tianhai</x:v>
+      </x:c>
+      <x:c r="B32" s="15" t="str">
+        <x:v>tars_a1</x:v>
+      </x:c>
+      <x:c r="C32" s="15" t="str">
+        <x:v>客户官方新闻</x:v>
+      </x:c>
+      <x:c r="D32" s="15" t="str">
+        <x:v>天海电子与它石智航战略合作</x:v>
+      </x:c>
+      <x:c r="E32" s="15" t="str">
+        <x:v>https://www.thb.com.cn/content/details_17_319668.html</x:v>
+      </x:c>
+      <x:c r="F32" s="15" t="str">
+        <x:v>2026-06-28</x:v>
+      </x:c>
+      <x:c r="G32" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H32" s="15" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="I32" s="15" t="str">
+        <x:v>确认汽车线束联合产线与近半年联合攻坚</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="42" customHeight="1">
+      <x:c r="A33" s="15" t="str">
+        <x:v>src_tars_shanghai</x:v>
+      </x:c>
+      <x:c r="B33" s="15" t="str">
+        <x:v>tars_a1</x:v>
+      </x:c>
+      <x:c r="C33" s="15" t="str">
+        <x:v>政府官方信息</x:v>
+      </x:c>
+      <x:c r="D33" s="15" t="str">
+        <x:v>它石智航产业化闭环</x:v>
+      </x:c>
+      <x:c r="E33" s="15" t="str">
+        <x:v>https://www.sheitc.sh.gov.cn/zxxx/20260710/480d32461ca145e3bf067ce67dc6c203.html</x:v>
+      </x:c>
+      <x:c r="F33" s="15" t="str">
+        <x:v>2026-07-10</x:v>
+      </x:c>
+      <x:c r="G33" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H33" s="15" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="I33" s="15" t="str">
+        <x:v>披露安波福百台计划、33类场景、46工位和DexHand</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="42" customHeight="1">
+      <x:c r="A34" s="15" t="str">
+        <x:v>src_tars_guinness</x:v>
+      </x:c>
+      <x:c r="B34" s="15" t="str">
+        <x:v>tars_a1</x:v>
+      </x:c>
+      <x:c r="C34" s="15" t="str">
+        <x:v>独立纪录机构</x:v>
+      </x:c>
+      <x:c r="D34" s="15" t="str">
+        <x:v>Most sub-millimeter wire harness assembled by a robot in one hour</x:v>
+      </x:c>
+      <x:c r="E34" s="15" t="str">
+        <x:v>https://guinnessworldrecords.com.br/world-records/782788-most-sub-millimeter-wire-harness-assembled-by-a-robot-in-one-hour</x:v>
+      </x:c>
+      <x:c r="F34" s="15" t="str"/>
+      <x:c r="G34" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H34" s="15" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="I34" s="15" t="str">
+        <x:v>确认一小时105次亚毫米线束装配纪录</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="42" customHeight="1">
+      <x:c r="A35" s="15" t="str">
+        <x:v>src_tars_internal</x:v>
+      </x:c>
+      <x:c r="B35" s="15" t="str">
+        <x:v>tars_a1</x:v>
+      </x:c>
+      <x:c r="C35" s="15" t="str">
+        <x:v>内部沟通</x:v>
+      </x:c>
+      <x:c r="D35" s="15" t="str">
+        <x:v>它石线束部署与工程问题纪要</x:v>
+      </x:c>
+      <x:c r="E35" s="15" t="str">
+        <x:v>conversation-context:2026-09-15</x:v>
+      </x:c>
+      <x:c r="F35" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="G35" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H35" s="15" t="str">
+        <x:v>待核验</x:v>
+      </x:c>
+      <x:c r="I35" s="15" t="str">
+        <x:v>反馈百台部署尚未达到要求并存在臂展、工装耗材、夹爪和MES依赖问题</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:I1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re134595142734ffa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a5ac16dabe9421a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add model gallery and replace Astribot S1 with T1
</commit_message>
<xml_diff>
--- a/outputs/机器人本体产品主表.xlsx
+++ b/outputs/机器人本体产品主表.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="决策摘要" sheetId="1" r:id="Rc6adbc6eae404cd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="场景评分" sheetId="2" r:id="Rad89cee4aa3d4cc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数主表" sheetId="3" r:id="R614e916d26b44e97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题清单" sheetId="4" r:id="R448bd1bface44fd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源证据" sheetId="5" r:id="R5f975c33ac3642b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="决策摘要" sheetId="1" r:id="R3ed96af3fcb64d1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="型号图示" sheetId="2" r:id="Ra0efeb1d15634d72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="场景评分" sheetId="3" r:id="R309e999abf524a6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数主表" sheetId="4" r:id="Rda6d8609b6234339"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题清单" sheetId="5" r:id="Rc18e434436c242e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源证据" sheetId="6" r:id="R8576dac86e3841f5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +22,7 @@
     <x:numFmt numFmtId="200" formatCode="0.00"/>
     <x:numFmt numFmtId="201" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -53,6 +54,18 @@
       <x:i/>
       <x:sz val="11"/>
       <x:color rgb="FF17365D"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="9"/>
+      <x:color rgb="FF6B7280"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
@@ -101,7 +114,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="28">
+  <x:cellXfs count="35">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -140,22 +153,39 @@
     <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
   </x:cellXfs>
@@ -231,6 +261,335 @@
     </x:dxf>
   </x:dxfs>
 </x:styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2333625" cy="1809750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="bac3d4ac-6310-4050-9783-14cfdba677ae"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R66cdb46197e146f7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2333625" cy="1809750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="f150938f-c0ce-49a7-866c-0ced09993435"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R06cb6e2fe5f34865"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2333625" cy="1809750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="b014cd1a-00ce-4f13-bdf2-b331697cc429"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7ee2b1508e5f40aa"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2333625" cy="1809750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="6ea4bc63-c241-40a2-a958-92d82d4122c2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2d0314bcdd0a49d0"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2333625" cy="1809750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="64a8a201-4279-4c15-b819-f08d78405f5e"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R032b736719cc4d96"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2333625" cy="1809750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="d56e322e-82f1-47d4-bb80-c94e1043b0e7"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6b544f7a2b3048f9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2333625" cy="1809750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="576a465f-5405-4978-beec-4e5548e5b1aa"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R07a47e47521b447a"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2333625" cy="1809750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="8a13efc3-8166-4539-8085-0c43ca22eefc"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0e9fff79102340e8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2333625" cy="1809750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="3eb2d835-326f-4a45-951f-22b66f5a91d8"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1c32660de22244be"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2333625" cy="1809750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="e84268cf-7b5c-4f24-80c7-19c313984720"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rabef248c63fd4c3f"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2333625" cy="1809750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="32a03535-4485-4296-a516-8190d9315295"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3dec1176d8b5473d"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2333625" cy="1809750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="5475ec6d-a94e-476b-a43e-aab0ba7284a0"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R71706e1d61cf4963"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -318,7 +677,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EvidenceSources" displayName="EvidenceSources" ref="A3:I35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EvidenceSources" displayName="EvidenceSources" ref="A3:I37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="source_id"/>
     <x:tableColumn id="2" name="model_id"/>
@@ -679,22 +1038,22 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B8" s="15" t="str">
-        <x:v>星尘</x:v>
+        <x:v>Boston Dynamics</x:v>
       </x:c>
       <x:c r="C8" s="15" t="str">
-        <x:v>Astribot S1</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="D8" s="16" t="n">
-        <x:v>3.95</x:v>
+        <x:v>3.85</x:v>
       </x:c>
       <x:c r="E8" s="15" t="str">
-        <x:v>通过待实测</x:v>
+        <x:v>待实测</x:v>
       </x:c>
       <x:c r="F8" s="15" t="str">
         <x:v>条件 POC</x:v>
       </x:c>
       <x:c r="G8" s="15" t="str">
-        <x:v>论文确认全向底盘；量产配置、接口和工业认证资料不足</x:v>
+        <x:v>工业可靠性负载和工作空间领先；但双足连续贴线横移、采购与集成开放性待确认</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="32" customHeight="1">
@@ -702,13 +1061,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B9" s="15" t="str">
-        <x:v>Boston Dynamics</x:v>
+        <x:v>Figure AI</x:v>
       </x:c>
       <x:c r="C9" s="15" t="str">
-        <x:v>Atlas</x:v>
+        <x:v>Figure 03</x:v>
       </x:c>
       <x:c r="D9" s="16" t="n">
-        <x:v>3.85</x:v>
+        <x:v>3.8000000000000003</x:v>
       </x:c>
       <x:c r="E9" s="15" t="str">
         <x:v>待实测</x:v>
@@ -717,7 +1076,7 @@
         <x:v>条件 POC</x:v>
       </x:c>
       <x:c r="G9" s="15" t="str">
-        <x:v>工业可靠性负载和工作空间领先；但双足连续贴线横移、采购与集成开放性待确认</x:v>
+        <x:v>触觉手和量产设计突出；无公开SDK且双足横移节拍与精度未披露</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="32" customHeight="1">
@@ -725,22 +1084,22 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B10" s="15" t="str">
-        <x:v>Figure AI</x:v>
+        <x:v>智动力</x:v>
       </x:c>
       <x:c r="C10" s="15" t="str">
-        <x:v>Figure 03</x:v>
+        <x:v>D1 擎骏系列</x:v>
       </x:c>
       <x:c r="D10" s="16" t="n">
-        <x:v>3.8000000000000003</x:v>
+        <x:v>3.8</x:v>
       </x:c>
       <x:c r="E10" s="15" t="str">
-        <x:v>待实测</x:v>
+        <x:v>通过待实测</x:v>
       </x:c>
       <x:c r="F10" s="15" t="str">
         <x:v>条件 POC</x:v>
       </x:c>
       <x:c r="G10" s="15" t="str">
-        <x:v>触觉手和量产设计突出；无公开SDK且双足横移节拍与精度未披露</x:v>
+        <x:v>四轮四转明确支持蟹行；整机重且精度和力控证据不足</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="32" customHeight="1">
@@ -748,22 +1107,22 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B11" s="15" t="str">
-        <x:v>智动力</x:v>
+        <x:v>它石智航</x:v>
       </x:c>
       <x:c r="C11" s="15" t="str">
-        <x:v>D1 擎骏系列</x:v>
+        <x:v>TARS A1</x:v>
       </x:c>
       <x:c r="D11" s="16" t="n">
-        <x:v>3.8</x:v>
+        <x:v>3.6500000000000004</x:v>
       </x:c>
       <x:c r="E11" s="15" t="str">
-        <x:v>通过待实测</x:v>
+        <x:v>待确认</x:v>
       </x:c>
       <x:c r="F11" s="15" t="str">
         <x:v>条件 POC</x:v>
       </x:c>
       <x:c r="G11" s="15" t="str">
-        <x:v>四轮四转明确支持蟹行；整机重且精度和力控证据不足</x:v>
+        <x:v>线束任务证据最强；底盘轮型接口参数和规模部署验收数据未公开且内部反馈仍有差距</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="32" customHeight="1">
@@ -771,22 +1130,22 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B12" s="15" t="str">
-        <x:v>它石智航</x:v>
+        <x:v>逐际动力</x:v>
       </x:c>
       <x:c r="C12" s="15" t="str">
-        <x:v>TARS A1</x:v>
+        <x:v>LimX Oli EDU</x:v>
       </x:c>
       <x:c r="D12" s="16" t="n">
-        <x:v>3.6500000000000004</x:v>
+        <x:v>3.3499999999999996</x:v>
       </x:c>
       <x:c r="E12" s="15" t="str">
-        <x:v>待确认</x:v>
+        <x:v>待实测</x:v>
       </x:c>
       <x:c r="F12" s="15" t="str">
-        <x:v>条件 POC</x:v>
+        <x:v>补齐资料后再评估</x:v>
       </x:c>
       <x:c r="G12" s="15" t="str">
-        <x:v>线束任务证据最强；底盘轮型接口参数和规模部署验收数据未公开且内部反馈仍有差距</x:v>
+        <x:v>开放开发工具链和全尺寸工作空间较好；双足贴线横移、精度和工业认证需验证</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="32" customHeight="1">
@@ -794,22 +1153,22 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B13" s="15" t="str">
-        <x:v>逐际动力</x:v>
+        <x:v>星尘</x:v>
       </x:c>
       <x:c r="C13" s="15" t="str">
-        <x:v>LimX Oli EDU</x:v>
+        <x:v>Astribot T1</x:v>
       </x:c>
       <x:c r="D13" s="16" t="n">
-        <x:v>3.3499999999999996</x:v>
+        <x:v>3.2</x:v>
       </x:c>
       <x:c r="E13" s="15" t="str">
-        <x:v>待实测</x:v>
+        <x:v>待确认</x:v>
       </x:c>
       <x:c r="F13" s="15" t="str">
         <x:v>补齐资料后再评估</x:v>
       </x:c>
       <x:c r="G13" s="15" t="str">
-        <x:v>开放开发工具链和全尺寸工作空间较好；双足贴线横移、精度和工业认证需验证</x:v>
+        <x:v>紧凑轮式底盘但轮系和蟹行能力未公开；绳驱柔性和量产进展较好，精度与SDK量化不足</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="32" customHeight="1">
@@ -1015,6 +1374,227 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="3" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="3" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="3" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="5" t="str">
+        <x:v>当前评比型号图示｜仅用于型号识别，参数与配置以来源证据为准</x:v>
+      </x:c>
+      <x:c r="B1" s="5"/>
+      <x:c r="C1" s="5"/>
+      <x:c r="D1" s="5"/>
+      <x:c r="E1" s="5"/>
+      <x:c r="F1" s="5"/>
+      <x:c r="G1" s="1"/>
+      <x:c r="H1" s="1"/>
+      <x:c r="I1" s="1"/>
+      <x:c r="J1" s="1"/>
+      <x:c r="K1" s="1"/>
+      <x:c r="L1" s="1"/>
+      <x:c r="M1" s="1"/>
+      <x:c r="N1" s="1"/>
+      <x:c r="O1" s="1"/>
+      <x:c r="P1" s="1"/>
+      <x:c r="Q1" s="1"/>
+      <x:c r="R1" s="1"/>
+      <x:c r="S1" s="1"/>
+      <x:c r="T1" s="1"/>
+      <x:c r="U1" s="1"/>
+      <x:c r="V1" s="1"/>
+      <x:c r="W1" s="1"/>
+      <x:c r="X1" s="1"/>
+      <x:c r="Y1" s="1"/>
+      <x:c r="Z1" s="1"/>
+      <x:c r="AA1" s="1"/>
+      <x:c r="AB1" s="1"/>
+      <x:c r="AC1" s="1"/>
+      <x:c r="AD1" s="1"/>
+      <x:c r="AE1" s="1"/>
+      <x:c r="AF1" s="1"/>
+      <x:c r="AG1" s="1"/>
+      <x:c r="AH1" s="1"/>
+      <x:c r="AI1" s="1"/>
+      <x:c r="AJ1" s="1"/>
+      <x:c r="AK1" s="1"/>
+      <x:c r="AL1" s="1"/>
+      <x:c r="AM1" s="1"/>
+      <x:c r="AN1" s="1"/>
+      <x:c r="AO1" s="1"/>
+      <x:c r="AP1" s="1"/>
+      <x:c r="AQ1" s="1"/>
+      <x:c r="AR1" s="1"/>
+      <x:c r="AS1" s="1"/>
+      <x:c r="AT1" s="1"/>
+      <x:c r="AU1" s="1"/>
+      <x:c r="AV1" s="1"/>
+      <x:c r="AW1" s="1"/>
+      <x:c r="AX1" s="1"/>
+      <x:c r="AY1" s="1"/>
+      <x:c r="AZ1" s="1"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="21" t="str">
+        <x:v>图片来源和本地文件映射见 data/images.csv；图片版权归原厂商或原发布方。</x:v>
+      </x:c>
+      <x:c r="B2" s="21" t="str"/>
+      <x:c r="C2" s="21" t="str"/>
+      <x:c r="D2" s="21" t="str"/>
+      <x:c r="E2" s="21" t="str"/>
+      <x:c r="F2" s="21" t="str"/>
+    </x:row>
+    <x:row r="3" ht="18" customHeight="1"/>
+    <x:row r="4" ht="18" customHeight="1">
+      <x:c r="A4" s="25" t="str">
+        <x:v>AgiBot 精灵G2</x:v>
+      </x:c>
+      <x:c r="C4" s="25" t="str">
+        <x:v>Astribot T1</x:v>
+      </x:c>
+      <x:c r="E4" s="25" t="str">
+        <x:v>D1 擎骏系列</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="18" customHeight="1"/>
+    <x:row r="6" ht="18" customHeight="1"/>
+    <x:row r="7" ht="18" customHeight="1"/>
+    <x:row r="8" ht="18" customHeight="1"/>
+    <x:row r="9" ht="18" customHeight="1"/>
+    <x:row r="10" ht="18" customHeight="1"/>
+    <x:row r="11" ht="18" customHeight="1"/>
+    <x:row r="12" ht="18" customHeight="1"/>
+    <x:row r="13" ht="18" customHeight="1"/>
+    <x:row r="14" ht="18" customHeight="1"/>
+    <x:row r="15" ht="18" customHeight="1">
+      <x:c r="A15" s="27" t="str">
+        <x:v>官方网站</x:v>
+      </x:c>
+      <x:c r="C15" s="27" t="str">
+        <x:v>官方网站</x:v>
+      </x:c>
+      <x:c r="E15" s="27" t="str">
+        <x:v>供应商PDF</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="18" customHeight="1"/>
+    <x:row r="17" ht="18" customHeight="1">
+      <x:c r="A17" s="25" t="str">
+        <x:v>JUNO2-SD 龙骏系列</x:v>
+      </x:c>
+      <x:c r="C17" s="25" t="str">
+        <x:v>Unitree G1-D 旗舰版</x:v>
+      </x:c>
+      <x:c r="E17" s="25" t="str">
+        <x:v>Atlas</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="18" customHeight="1"/>
+    <x:row r="19" ht="18" customHeight="1"/>
+    <x:row r="20" ht="18" customHeight="1"/>
+    <x:row r="21" ht="18" customHeight="1"/>
+    <x:row r="22" ht="18" customHeight="1"/>
+    <x:row r="23" ht="18" customHeight="1"/>
+    <x:row r="24" ht="18" customHeight="1"/>
+    <x:row r="25" ht="18" customHeight="1"/>
+    <x:row r="26" ht="18" customHeight="1"/>
+    <x:row r="27" ht="18" customHeight="1"/>
+    <x:row r="28" ht="18" customHeight="1">
+      <x:c r="A28" s="27" t="str">
+        <x:v>供应商PDF</x:v>
+      </x:c>
+      <x:c r="C28" s="27" t="str">
+        <x:v>官方网站</x:v>
+      </x:c>
+      <x:c r="E28" s="27" t="str">
+        <x:v>官方网站</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="18" customHeight="1"/>
+    <x:row r="30" ht="18" customHeight="1">
+      <x:c r="A30" s="25" t="str">
+        <x:v>Figure 03</x:v>
+      </x:c>
+      <x:c r="C30" s="25" t="str">
+        <x:v>Optimus</x:v>
+      </x:c>
+      <x:c r="E30" s="25" t="str">
+        <x:v>LimX Oli EDU</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="18" customHeight="1"/>
+    <x:row r="32" ht="18" customHeight="1"/>
+    <x:row r="33" ht="18" customHeight="1"/>
+    <x:row r="34" ht="18" customHeight="1"/>
+    <x:row r="35" ht="18" customHeight="1"/>
+    <x:row r="36" ht="18" customHeight="1"/>
+    <x:row r="37" ht="18" customHeight="1"/>
+    <x:row r="38" ht="18" customHeight="1"/>
+    <x:row r="39" ht="18" customHeight="1"/>
+    <x:row r="40" ht="18" customHeight="1"/>
+    <x:row r="41" ht="18" customHeight="1">
+      <x:c r="A41" s="27" t="str">
+        <x:v>官方网站</x:v>
+      </x:c>
+      <x:c r="C41" s="27" t="str">
+        <x:v>第三方型号图库</x:v>
+      </x:c>
+      <x:c r="E41" s="27" t="str">
+        <x:v>经销商产品图</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="18" customHeight="1"/>
+    <x:row r="43" ht="18" customHeight="1">
+      <x:c r="A43" s="25" t="str">
+        <x:v>TRON 2 双臂形态</x:v>
+      </x:c>
+      <x:c r="C43" s="25" t="str">
+        <x:v>Galaxea R1 Pro 2026</x:v>
+      </x:c>
+      <x:c r="E43" s="25" t="str">
+        <x:v>TARS A1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="18" customHeight="1"/>
+    <x:row r="45" ht="18" customHeight="1"/>
+    <x:row r="46" ht="18" customHeight="1"/>
+    <x:row r="47" ht="18" customHeight="1"/>
+    <x:row r="48" ht="18" customHeight="1"/>
+    <x:row r="49" ht="18" customHeight="1"/>
+    <x:row r="50" ht="18" customHeight="1"/>
+    <x:row r="51" ht="18" customHeight="1"/>
+    <x:row r="52" ht="18" customHeight="1"/>
+    <x:row r="53" ht="18" customHeight="1"/>
+    <x:row r="54" ht="18" customHeight="1">
+      <x:c r="A54" s="27" t="str">
+        <x:v>第三方型号图库</x:v>
+      </x:c>
+      <x:c r="C54" s="27" t="str">
+        <x:v>官方网站</x:v>
+      </x:c>
+      <x:c r="E54" s="27" t="str">
+        <x:v>政府公开信息</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="18" customHeight="1"/>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc34418df3938428d"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1090,48 +1670,48 @@
       <x:c r="AZ1" s="1"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="24" t="str">
+      <x:c r="A3" s="31" t="str">
         <x:v>评分维度</x:v>
       </x:c>
-      <x:c r="B3" s="24" t="str">
+      <x:c r="B3" s="31" t="str">
         <x:v>底盘全向与贴线能力</x:v>
       </x:c>
-      <x:c r="C3" s="24" t="str">
+      <x:c r="C3" s="31" t="str">
         <x:v>双臂与躯干工作空间</x:v>
       </x:c>
-      <x:c r="D3" s="24" t="str">
+      <x:c r="D3" s="31" t="str">
         <x:v>力控与柔顺能力</x:v>
       </x:c>
-      <x:c r="E3" s="24" t="str">
+      <x:c r="E3" s="31" t="str">
         <x:v>定位与视觉闭环</x:v>
       </x:c>
-      <x:c r="F3" s="24" t="str">
+      <x:c r="F3" s="31" t="str">
         <x:v>SDK与末端接口成熟度</x:v>
       </x:c>
-      <x:c r="G3" s="24" t="str">
+      <x:c r="G3" s="31" t="str">
         <x:v>工业可靠性与维护</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="26" t="str">
+      <x:c r="A4" s="33" t="str">
         <x:v>权重</x:v>
       </x:c>
-      <x:c r="B4" s="27" t="n">
+      <x:c r="B4" s="34" t="n">
         <x:v>0.25</x:v>
       </x:c>
-      <x:c r="C4" s="27" t="n">
+      <x:c r="C4" s="34" t="n">
         <x:v>0.15</x:v>
       </x:c>
-      <x:c r="D4" s="27" t="n">
+      <x:c r="D4" s="34" t="n">
         <x:v>0.2</x:v>
       </x:c>
-      <x:c r="E4" s="27" t="n">
+      <x:c r="E4" s="34" t="n">
         <x:v>0.15</x:v>
       </x:c>
-      <x:c r="F4" s="27" t="n">
+      <x:c r="F4" s="34" t="n">
         <x:v>0.1</x:v>
       </x:c>
-      <x:c r="G4" s="27" t="n">
+      <x:c r="G4" s="34" t="n">
         <x:v>0.15</x:v>
       </x:c>
     </x:row>
@@ -1224,42 +1804,42 @@
         <x:v>星尘</x:v>
       </x:c>
       <x:c r="B8" s="15" t="str">
-        <x:v>Astribot S1</x:v>
+        <x:v>Astribot T1</x:v>
       </x:c>
       <x:c r="C8" s="15" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="D8" s="15" t="str">
-        <x:v>通过待实测</x:v>
+        <x:v>待确认</x:v>
       </x:c>
       <x:c r="E8" s="15" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F8" s="15" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G8" s="15" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H8" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I8" s="15" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="I8" s="15" t="n">
-        <x:v>3</x:v>
-      </x:c>
       <x:c r="J8" s="15" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="K8" s="16" t="n">
         <x:f>IF(C8&lt;&gt;"是","",SUMPRODUCT(E8:J8,$B$4:$G$4))</x:f>
-        <x:v>3.95</x:v>
+        <x:v>3.2</x:v>
       </x:c>
       <x:c r="L8" s="15" t="str">
         <x:f>IF(C8&lt;&gt;"是","不参与移动本体排名",IF(D8="不通过","不进入布线POC",IF(K8&gt;=4.2,"优先POC",IF(K8&gt;=3.5,"条件POC","补齐资料后再评估"))))</x:f>
-        <x:v>条件POC</x:v>
+        <x:v>补齐资料后再评估</x:v>
       </x:c>
       <x:c r="M8" s="15" t="str">
-        <x:v>论文确认全向底盘；量产配置、接口和工业认证资料不足</x:v>
+        <x:v>紧凑轮式底盘但轮系和蟹行能力未公开；绳驱柔性和量产进展较好，精度与SDK量化不足</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -1937,12 +2517,12 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R728af8975e604a66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbe4832f0df04260"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2265,93 +2845,75 @@
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="15" t="str">
-        <x:v>astribot_s1</x:v>
+        <x:v>astribot_t1</x:v>
       </x:c>
       <x:c r="B5" s="15" t="str">
         <x:v>星尘</x:v>
       </x:c>
       <x:c r="C5" s="15" t="str">
-        <x:v>Astribot S1</x:v>
+        <x:v>Astribot T1</x:v>
       </x:c>
       <x:c r="D5" s="15" t="str">
         <x:v>移动双臂本体</x:v>
       </x:c>
       <x:c r="E5" s="15" t="str">
-        <x:v>科研/行业共创</x:v>
+        <x:v>量产/发货</x:v>
       </x:c>
       <x:c r="F5" s="15" t="n">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="G5" s="15" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H5" s="15" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="I5" s="15" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J5" s="15" t="n">
-        <x:v>3</x:v>
-      </x:c>
+      <x:c r="G5" s="15"/>
+      <x:c r="H5" s="15"/>
+      <x:c r="I5" s="15"/>
+      <x:c r="J5" s="15"/>
       <x:c r="K5" s="15" t="str">
-        <x:v>三自由度全向移动底盘</x:v>
+        <x:v>紧凑轮式底盘（轮系未公开）</x:v>
       </x:c>
       <x:c r="L5" s="15" t="str">
-        <x:v>是</x:v>
+        <x:v>待确认</x:v>
       </x:c>
       <x:c r="M5" s="15"/>
       <x:c r="N5" s="15" t="n">
-        <x:v>1700</x:v>
+        <x:v>1550</x:v>
       </x:c>
       <x:c r="O5" s="15" t="n">
-        <x:v>1700</x:v>
+        <x:v>1550</x:v>
       </x:c>
       <x:c r="P5" s="15"/>
       <x:c r="Q5" s="15"/>
       <x:c r="R5" s="15" t="n">
-        <x:v>80</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="S5" s="15"/>
-      <x:c r="T5" s="15" t="n">
-        <x:v>1940</x:v>
-      </x:c>
+      <x:c r="T5" s="15"/>
       <x:c r="U5" s="15" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="V5" s="15"/>
       <x:c r="W5" s="15"/>
       <x:c r="X5" s="15"/>
-      <x:c r="Y5" s="15" t="str">
-        <x:v>0-2.0</x:v>
-      </x:c>
-      <x:c r="Z5" s="15" t="n">
-        <x:v>0.1</x:v>
-      </x:c>
+      <x:c r="Y5" s="15" t="str"/>
+      <x:c r="Z5" s="15"/>
       <x:c r="AA5" s="15"/>
       <x:c r="AB5" s="15" t="str">
-        <x:v>强调柔顺与全身操作，公开量化不足</x:v>
+        <x:v>绳驱柔性；碰撞卸力（控制与传感指标未公开）</x:v>
       </x:c>
       <x:c r="AC5" s="15"/>
       <x:c r="AD5" s="15"/>
-      <x:c r="AE5" s="15" t="str">
-        <x:v>未公开</x:v>
-      </x:c>
-      <x:c r="AF5" s="15" t="str">
-        <x:v>4-6</x:v>
-      </x:c>
+      <x:c r="AE5" s="15" t="str"/>
+      <x:c r="AF5" s="15" t="str"/>
       <x:c r="AG5" s="15" t="str"/>
       <x:c r="AH5" s="15" t="str">
-        <x:v>平行二指夹爪</x:v>
+        <x:v>支持多样末端配置与更换</x:v>
       </x:c>
       <x:c r="AI5" s="15" t="str">
-        <x:v>API；VR遥操作；仿真与训练工具链</x:v>
+        <x:v>末端与算力背包扩展接口；自动回充；快捷换电（协议未公开）</x:v>
       </x:c>
       <x:c r="AJ5" s="15" t="str">
-        <x:v>官网+研发论文</x:v>
+        <x:v>官网+政府及媒体报道</x:v>
       </x:c>
       <x:c r="AK5" s="15" t="str">
-        <x:v>底盘轮型、速度、定位精度及工业认证未公开</x:v>
+        <x:v>8.99万元起；底盘是否全向、移动与操作精度、SDK协议、续航和工业认证未公开</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
@@ -3585,12 +4147,12 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab0e2da811f447fa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47646d5dd2334ada"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -3842,7 +4404,7 @@
         <x:v>星尘</x:v>
       </x:c>
       <x:c r="C9" s="15" t="str">
-        <x:v>S1</x:v>
+        <x:v>T1</x:v>
       </x:c>
       <x:c r="D9" s="15" t="str">
         <x:v>P0</x:v>
@@ -3851,10 +4413,10 @@
         <x:v>底盘</x:v>
       </x:c>
       <x:c r="F9" s="15" t="str">
-        <x:v>全向底盘的轮型、最大横移速度、定位精度和航向误差是多少</x:v>
+        <x:v>紧凑轮式底盘采用什么轮系，是否支持保持机身朝向纯横移/蟹行，最大横移速度、定位精度和航向误差是多少</x:v>
       </x:c>
       <x:c r="G9" s="15" t="str">
-        <x:v>论文只确认3DOF全向底盘</x:v>
+        <x:v>公开资料只说明紧凑轮式底盘和自动回充，未证明全向能力</x:v>
       </x:c>
       <x:c r="H9" s="15" t="str">
         <x:v>待供应商回复</x:v>
@@ -3870,19 +4432,19 @@
         <x:v>星尘</x:v>
       </x:c>
       <x:c r="C10" s="15" t="str">
-        <x:v>S1</x:v>
+        <x:v>T1</x:v>
       </x:c>
       <x:c r="D10" s="15" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="E10" s="15" t="str">
-        <x:v>力控</x:v>
+        <x:v>精度与力控</x:v>
       </x:c>
       <x:c r="F10" s="15" t="str">
-        <x:v>关节或末端力传感器的分辨率、采样率和阻抗控制接口是什么</x:v>
+        <x:v>机械臂重复定位精度、整机移动后TCP误差、力传感器分辨率/采样率及阻抗控制接口分别是多少</x:v>
       </x:c>
       <x:c r="G10" s="15" t="str">
-        <x:v>官网未公开量化参数</x:v>
+        <x:v>仅公开绳驱柔性和碰撞卸力，未给量化精度与力控指标</x:v>
       </x:c>
       <x:c r="H10" s="15" t="str">
         <x:v>待供应商回复</x:v>
@@ -3898,19 +4460,19 @@
         <x:v>星尘</x:v>
       </x:c>
       <x:c r="C11" s="15" t="str">
-        <x:v>S1</x:v>
+        <x:v>T1</x:v>
       </x:c>
       <x:c r="D11" s="15" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="E11" s="15" t="str">
         <x:v>接口</x:v>
       </x:c>
       <x:c r="F11" s="15" t="str">
-        <x:v>SDK协议、控制频率、ROS版本和末端供电通信接口是什么</x:v>
+        <x:v>SDK协议、控制频率、ROS版本、末端供电通信和算力背包接口定义是什么</x:v>
       </x:c>
       <x:c r="G11" s="15" t="str">
-        <x:v>官网只说明提供API和工具链</x:v>
+        <x:v>公开资料只说明支持软硬件扩展、末端与算力背包更换</x:v>
       </x:c>
       <x:c r="H11" s="15" t="str">
         <x:v>待供应商回复</x:v>
@@ -3926,7 +4488,7 @@
         <x:v>星尘</x:v>
       </x:c>
       <x:c r="C12" s="15" t="str">
-        <x:v>S1</x:v>
+        <x:v>T1</x:v>
       </x:c>
       <x:c r="D12" s="15" t="str">
         <x:v>P1</x:v>
@@ -3935,10 +4497,10 @@
         <x:v>工业安全</x:v>
       </x:c>
       <x:c r="F12" s="15" t="str">
-        <x:v>IP等级、安全认证、MTBF和连续运行数据是什么</x:v>
+        <x:v>电池容量与续航、换电/回充节拍、IP等级、安全认证、MTBF和连续运行数据是什么</x:v>
       </x:c>
       <x:c r="G12" s="15" t="str">
-        <x:v>公开资料未披露</x:v>
+        <x:v>公开资料未披露量化指标</x:v>
       </x:c>
       <x:c r="H12" s="15" t="str">
         <x:v>待供应商回复</x:v>
@@ -4609,12 +5171,12 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01a047f617b34a1b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfceb751f894a4c15"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -4631,7 +5193,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>来源证据登记｜内部文件仅登记名称，不随仓库上传</x:v>
+        <x:v>来源证据登记｜原始供应商文件按仓库策略归档</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -4727,8 +5289,9 @@
       <x:c r="D4" s="15" t="str">
         <x:v>智元精灵G2产品用户手册</x:v>
       </x:c>
-      <x:c r="E4" s="15" t="str">
-        <x:v>https://www.agibot.com.cn/filepage/362.html</x:v>
+      <x:c r="E4" s="15" t="e">
+        <x:f>HYPERLINK("https://www.agibot.com.cn/filepage/362.html","https://www.agibot.com.cn/filepage/362.html")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://www.agibot.com.cn/filepage/362.html, friendlyName=https://www.agibot.com.cn/filepage/362.html</x:v>
       </x:c>
       <x:c r="F4" s="15" t="str">
         <x:v>2026-04-28</x:v>
@@ -4745,19 +5308,20 @@
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
       <x:c r="A5" s="15" t="str">
-        <x:v>src_astribot_s1_official</x:v>
+        <x:v>src_astribot_t1_home</x:v>
       </x:c>
       <x:c r="B5" s="15" t="str">
-        <x:v>astribot_s1</x:v>
+        <x:v>astribot_t1</x:v>
       </x:c>
       <x:c r="C5" s="15" t="str">
         <x:v>官方网站</x:v>
       </x:c>
       <x:c r="D5" s="15" t="str">
-        <x:v>星尘智能S1产品页</x:v>
-      </x:c>
-      <x:c r="E5" s="15" t="str">
-        <x:v>https://www.astribot.com/product/</x:v>
+        <x:v>星尘智能首页 T1 发布信息</x:v>
+      </x:c>
+      <x:c r="E5" s="15" t="e">
+        <x:f>HYPERLINK("https://www.astribot.com/","https://www.astribot.com/")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://www.astribot.com/, friendlyName=https://www.astribot.com/</x:v>
       </x:c>
       <x:c r="F5" s="15" t="str"/>
       <x:c r="G5" s="15" t="str">
@@ -4767,27 +5331,28 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="I5" s="15" t="str">
-        <x:v>包含操作性能和整机基础参数</x:v>
+        <x:v>确认T1型号与8.99万元起售价；官网尚无T1完整数据表</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="15" t="str">
-        <x:v>src_astribot_suite</x:v>
+        <x:v>src_astribot_t1_wuxi</x:v>
       </x:c>
       <x:c r="B6" s="15" t="str">
-        <x:v>astribot_s1</x:v>
+        <x:v>astribot_t1</x:v>
       </x:c>
       <x:c r="C6" s="15" t="str">
-        <x:v>研发论文</x:v>
+        <x:v>政府公开信息</x:v>
       </x:c>
       <x:c r="D6" s="15" t="str">
-        <x:v>Towards Human-level Intelligence via Human-like Whole-Body Manipulation</x:v>
-      </x:c>
-      <x:c r="E6" s="15" t="str">
-        <x:v>https://arxiv.org/abs/2507.17141</x:v>
+        <x:v>技术硬核价格亲民 多元场景显身手</x:v>
+      </x:c>
+      <x:c r="E6" s="15" t="e">
+        <x:f>HYPERLINK("https://www.wuxi.gov.cn/doc/2026/07/11/4803940.shtml","https://www.wuxi.gov.cn/doc/2026/07/11/4803940.shtml")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://www.wuxi.gov.cn/doc/2026/07/11/4803940.shtml, friendlyName=https://www.wuxi.gov.cn/doc/2026/07/11/4803940.shtml</x:v>
       </x:c>
       <x:c r="F6" s="15" t="str">
-        <x:v>2025-07-23</x:v>
+        <x:v>2026-07-11</x:v>
       </x:c>
       <x:c r="G6" s="15" t="str">
         <x:v>2026-09-15</x:v>
@@ -4796,132 +5361,140 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="I6" s="15" t="str">
-        <x:v>包含23自由度构成和三自由度全向底盘</x:v>
+        <x:v>确认无锡工厂量产下线、23自由度、单臂5kg、绳驱和底盘扩展接口</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="15" t="str">
-        <x:v>src_unitree_g1d</x:v>
+        <x:v>src_astribot_t1_sznews</x:v>
       </x:c>
       <x:c r="B7" s="15" t="str">
-        <x:v>unitree_g1d_flagship</x:v>
+        <x:v>astribot_t1</x:v>
       </x:c>
       <x:c r="C7" s="15" t="str">
-        <x:v>官方网站</x:v>
+        <x:v>地方官方媒体</x:v>
       </x:c>
       <x:c r="D7" s="15" t="str">
-        <x:v>Unitree G1-D产品参数</x:v>
-      </x:c>
-      <x:c r="E7" s="15" t="str">
-        <x:v>https://www.unitree.com/cn/mobile/G1-D/</x:v>
-      </x:c>
-      <x:c r="F7" s="15" t="str"/>
+        <x:v>煎牛排调酒做实验 星尘智能发布绳驱AI机器人T1</x:v>
+      </x:c>
+      <x:c r="E7" s="15" t="e">
+        <x:f>HYPERLINK("https://www.sznews.com/news/content/2026-05/27/content_32067943.htm","https://www.sznews.com/news/content/2026-05/27/content_32067943.htm")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://www.sznews.com/news/content/2026-05/27/content_32067943.htm, friendlyName=https://www.sznews.com/news/content/2026-05/27/content_32067943.htm</x:v>
+      </x:c>
+      <x:c r="F7" s="15" t="str">
+        <x:v>2026-05-27</x:v>
+      </x:c>
       <x:c r="G7" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
       <x:c r="H7" s="15" t="str">
-        <x:v>高</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="I7" s="15" t="str">
-        <x:v>同时覆盖旗舰版和通用版</x:v>
+        <x:v>确认155cm、约66kg、23自由度不含末端、单臂5kg、自动回充和快捷换电</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="15" t="str">
-        <x:v>src_unitree_g1d_std</x:v>
+        <x:v>src_astribot_t1_wrc</x:v>
       </x:c>
       <x:c r="B8" s="15" t="str">
-        <x:v>unitree_g1d_standard</x:v>
+        <x:v>astribot_t1</x:v>
       </x:c>
       <x:c r="C8" s="15" t="str">
-        <x:v>官方网站</x:v>
+        <x:v>行业展会官方信息</x:v>
       </x:c>
       <x:c r="D8" s="15" t="str">
-        <x:v>Unitree G1-D产品参数</x:v>
-      </x:c>
-      <x:c r="E8" s="15" t="str">
-        <x:v>https://www.unitree.com/cn/mobile/G1-D/</x:v>
-      </x:c>
-      <x:c r="F8" s="15" t="str"/>
+        <x:v>2026世界机器人大会星尘智能展品介绍</x:v>
+      </x:c>
+      <x:c r="E8" s="15" t="e">
+        <x:f>HYPERLINK("https://wrc.cie.org.cn/expo/company/441.html","https://wrc.cie.org.cn/expo/company/441.html")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://wrc.cie.org.cn/expo/company/441.html, friendlyName=https://wrc.cie.org.cn/expo/company/441.html</x:v>
+      </x:c>
+      <x:c r="F8" s="15" t="str">
+        <x:v>2026-08-19</x:v>
+      </x:c>
       <x:c r="G8" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
       <x:c r="H8" s="15" t="str">
-        <x:v>高</x:v>
+        <x:v>中高</x:v>
       </x:c>
       <x:c r="I8" s="15" t="str">
-        <x:v>通用版无主动底盘参数</x:v>
+        <x:v>确认轻量化机身、紧凑底盘、多样末端和软硬件扩展；未披露轮系</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="15" t="str">
-        <x:v>src_zdl_d1</x:v>
+        <x:v>src_unitree_g1d</x:v>
       </x:c>
       <x:c r="B9" s="15" t="str">
-        <x:v>zdl_d1</x:v>
+        <x:v>unitree_g1d_flagship</x:v>
       </x:c>
       <x:c r="C9" s="15" t="str">
-        <x:v>供应商PDF</x:v>
+        <x:v>官方网站</x:v>
       </x:c>
       <x:c r="D9" s="15" t="str">
-        <x:v>D1（擎骏系列）.pdf</x:v>
-      </x:c>
-      <x:c r="E9" s="15" t="str">
-        <x:v>sources/raw/01_智动力/D1（擎骏系列）.pdf</x:v>
+        <x:v>Unitree G1-D产品参数</x:v>
+      </x:c>
+      <x:c r="E9" s="15" t="e">
+        <x:f>HYPERLINK("https://www.unitree.com/cn/mobile/G1-D/","https://www.unitree.com/cn/mobile/G1-D/")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://www.unitree.com/cn/mobile/G1-D/, friendlyName=https://www.unitree.com/cn/mobile/G1-D/</x:v>
       </x:c>
       <x:c r="F9" s="15" t="str"/>
       <x:c r="G9" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
       <x:c r="H9" s="15" t="str">
-        <x:v>中</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="I9" s="15" t="str">
-        <x:v>供应商产品册，尚未实测</x:v>
+        <x:v>同时覆盖旗舰版和通用版</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="15" t="str">
-        <x:v>src_zdl_juno2</x:v>
+        <x:v>src_unitree_g1d_std</x:v>
       </x:c>
       <x:c r="B10" s="15" t="str">
-        <x:v>zdl_juno2</x:v>
+        <x:v>unitree_g1d_standard</x:v>
       </x:c>
       <x:c r="C10" s="15" t="str">
-        <x:v>供应商PDF</x:v>
+        <x:v>官方网站</x:v>
       </x:c>
       <x:c r="D10" s="15" t="str">
-        <x:v>JUNO2-SD（龙骏系列）.pdf</x:v>
-      </x:c>
-      <x:c r="E10" s="15" t="str">
-        <x:v>sources/raw/01_智动力/JUNO2-SD（龙骏系列）.pdf</x:v>
+        <x:v>Unitree G1-D产品参数</x:v>
+      </x:c>
+      <x:c r="E10" s="15" t="e">
+        <x:f>HYPERLINK("https://www.unitree.com/cn/mobile/G1-D/","https://www.unitree.com/cn/mobile/G1-D/")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://www.unitree.com/cn/mobile/G1-D/, friendlyName=https://www.unitree.com/cn/mobile/G1-D/</x:v>
       </x:c>
       <x:c r="F10" s="15" t="str"/>
       <x:c r="G10" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
       <x:c r="H10" s="15" t="str">
-        <x:v>中</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="I10" s="15" t="str">
-        <x:v>供应商产品册，尚未实测</x:v>
+        <x:v>通用版无主动底盘参数</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="15" t="str">
-        <x:v>src_zdl_juno1</x:v>
+        <x:v>src_zdl_d1</x:v>
       </x:c>
       <x:c r="B11" s="15" t="str">
-        <x:v>zdl_juno1</x:v>
+        <x:v>zdl_d1</x:v>
       </x:c>
       <x:c r="C11" s="15" t="str">
         <x:v>供应商PDF</x:v>
       </x:c>
       <x:c r="D11" s="15" t="str">
-        <x:v>JUNO1-P（智骏系列）.pdf</x:v>
+        <x:v>D1（擎骏系列）.pdf</x:v>
       </x:c>
       <x:c r="E11" s="15" t="str">
-        <x:v>sources/raw/01_智动力/JUNO1-P（智骏系列）.pdf</x:v>
+        <x:v>sources/raw/01_智动力/D1（擎骏系列）.pdf</x:v>
       </x:c>
       <x:c r="F11" s="15" t="str"/>
       <x:c r="G11" s="15" t="str">
@@ -4936,19 +5509,19 @@
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="15" t="str">
-        <x:v>src_zdl_l1</x:v>
+        <x:v>src_zdl_juno2</x:v>
       </x:c>
       <x:c r="B12" s="15" t="str">
-        <x:v>zdl_l1</x:v>
+        <x:v>zdl_juno2</x:v>
       </x:c>
       <x:c r="C12" s="15" t="str">
         <x:v>供应商PDF</x:v>
       </x:c>
       <x:c r="D12" s="15" t="str">
-        <x:v>L1（灵骏系列）.pdf</x:v>
+        <x:v>JUNO2-SD（龙骏系列）.pdf</x:v>
       </x:c>
       <x:c r="E12" s="15" t="str">
-        <x:v>sources/raw/01_智动力/L1（灵骏系列）.pdf</x:v>
+        <x:v>sources/raw/01_智动力/JUNO2-SD（龙骏系列）.pdf</x:v>
       </x:c>
       <x:c r="F12" s="15" t="str"/>
       <x:c r="G12" s="15" t="str">
@@ -4963,23 +5536,21 @@
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="15" t="str">
-        <x:v>src_zdl_z1</x:v>
+        <x:v>src_zdl_juno1</x:v>
       </x:c>
       <x:c r="B13" s="15" t="str">
-        <x:v>zdl_z1</x:v>
+        <x:v>zdl_juno1</x:v>
       </x:c>
       <x:c r="C13" s="15" t="str">
-        <x:v>供应商开发手册</x:v>
+        <x:v>供应商PDF</x:v>
       </x:c>
       <x:c r="D13" s="15" t="str">
-        <x:v>全尺寸人形机器人Z1开发手册 r26.6.md</x:v>
+        <x:v>JUNO1-P（智骏系列）.pdf</x:v>
       </x:c>
       <x:c r="E13" s="15" t="str">
-        <x:v>sources/raw/01_智动力/全尺寸人形机器人Z1开发手册 r26.6.md</x:v>
-      </x:c>
-      <x:c r="F13" s="15" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
+        <x:v>sources/raw/01_智动力/JUNO1-P（智骏系列）.pdf</x:v>
+      </x:c>
+      <x:c r="F13" s="15" t="str"/>
       <x:c r="G13" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
@@ -4987,24 +5558,24 @@
         <x:v>中</x:v>
       </x:c>
       <x:c r="I13" s="15" t="str">
-        <x:v>接口文档存在多项待澄清问题</x:v>
+        <x:v>供应商产品册，尚未实测</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="15" t="str">
-        <x:v>src_zdl_ha</x:v>
+        <x:v>src_zdl_l1</x:v>
       </x:c>
       <x:c r="B14" s="15" t="str">
-        <x:v>zdl_ha</x:v>
+        <x:v>zdl_l1</x:v>
       </x:c>
       <x:c r="C14" s="15" t="str">
         <x:v>供应商PDF</x:v>
       </x:c>
       <x:c r="D14" s="15" t="str">
-        <x:v>人形臂（HA系列）.pdf</x:v>
+        <x:v>L1（灵骏系列）.pdf</x:v>
       </x:c>
       <x:c r="E14" s="15" t="str">
-        <x:v>sources/raw/01_智动力/人形臂（HA系列）.pdf</x:v>
+        <x:v>sources/raw/01_智动力/L1（灵骏系列）.pdf</x:v>
       </x:c>
       <x:c r="F14" s="15" t="str"/>
       <x:c r="G14" s="15" t="str">
@@ -5014,26 +5585,28 @@
         <x:v>中</x:v>
       </x:c>
       <x:c r="I14" s="15" t="str">
-        <x:v>待纳入机械臂专项对比</x:v>
+        <x:v>供应商产品册，尚未实测</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="15" t="str">
-        <x:v>src_zdl_fa</x:v>
+        <x:v>src_zdl_z1</x:v>
       </x:c>
       <x:c r="B15" s="15" t="str">
-        <x:v>zdl_fa</x:v>
+        <x:v>zdl_z1</x:v>
       </x:c>
       <x:c r="C15" s="15" t="str">
-        <x:v>供应商PDF</x:v>
+        <x:v>供应商开发手册</x:v>
       </x:c>
       <x:c r="D15" s="15" t="str">
-        <x:v>桌面臂（FA系列）.pdf</x:v>
+        <x:v>全尺寸人形机器人Z1开发手册 r26.6.md</x:v>
       </x:c>
       <x:c r="E15" s="15" t="str">
-        <x:v>sources/raw/01_智动力/桌面臂（FA系列）.pdf</x:v>
-      </x:c>
-      <x:c r="F15" s="15" t="str"/>
+        <x:v>sources/raw/01_智动力/全尺寸人形机器人Z1开发手册 r26.6.md</x:v>
+      </x:c>
+      <x:c r="F15" s="15" t="str">
+        <x:v>2026-07-25</x:v>
+      </x:c>
       <x:c r="G15" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
@@ -5041,24 +5614,24 @@
         <x:v>中</x:v>
       </x:c>
       <x:c r="I15" s="15" t="str">
-        <x:v>待纳入机械臂专项对比</x:v>
+        <x:v>接口文档存在多项待澄清问题</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="15" t="str">
-        <x:v>src_flexiv_rizon4_manual</x:v>
+        <x:v>src_zdl_ha</x:v>
       </x:c>
       <x:c r="B16" s="15" t="str">
-        <x:v>flexiv_rizon4</x:v>
+        <x:v>zdl_ha</x:v>
       </x:c>
       <x:c r="C16" s="15" t="str">
         <x:v>供应商PDF</x:v>
       </x:c>
       <x:c r="D16" s="15" t="str">
-        <x:v>Rizon4 用户手册_V3.0_zh-CN.pdf</x:v>
+        <x:v>人形臂（HA系列）.pdf</x:v>
       </x:c>
       <x:c r="E16" s="15" t="str">
-        <x:v>sources/raw/02_非夕_Flexiv/01_Rizon_拂晓/Rizon4 用户手册_V3.0_zh-CN.pdf</x:v>
+        <x:v>sources/raw/01_智动力/人形臂（HA系列）.pdf</x:v>
       </x:c>
       <x:c r="F16" s="15" t="str"/>
       <x:c r="G16" s="15" t="str">
@@ -5073,23 +5646,21 @@
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="15" t="str">
-        <x:v>src_flexiv_rizon_datasheet</x:v>
+        <x:v>src_zdl_fa</x:v>
       </x:c>
       <x:c r="B17" s="15" t="str">
-        <x:v>flexiv_rizon</x:v>
+        <x:v>zdl_fa</x:v>
       </x:c>
       <x:c r="C17" s="15" t="str">
         <x:v>供应商PDF</x:v>
       </x:c>
       <x:c r="D17" s="15" t="str">
-        <x:v>拂晓(Rizon)机器人数据表_V2.0_202409.pdf</x:v>
+        <x:v>桌面臂（FA系列）.pdf</x:v>
       </x:c>
       <x:c r="E17" s="15" t="str">
-        <x:v>sources/raw/02_非夕_Flexiv/01_Rizon_拂晓/拂晓(Rizon)机器人数据表_V2.0_202409.pdf</x:v>
-      </x:c>
-      <x:c r="F17" s="15" t="str">
-        <x:v>2024-09</x:v>
-      </x:c>
+        <x:v>sources/raw/01_智动力/桌面臂（FA系列）.pdf</x:v>
+      </x:c>
+      <x:c r="F17" s="15" t="str"/>
       <x:c r="G17" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
@@ -5102,23 +5673,21 @@
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="15" t="str">
-        <x:v>src_flexiv_grav_manual</x:v>
+        <x:v>src_flexiv_rizon4_manual</x:v>
       </x:c>
       <x:c r="B18" s="15" t="str">
-        <x:v>flexiv_grav</x:v>
+        <x:v>flexiv_rizon4</x:v>
       </x:c>
       <x:c r="C18" s="15" t="str">
         <x:v>供应商PDF</x:v>
       </x:c>
       <x:c r="D18" s="15" t="str">
-        <x:v>星擎用户手册_V1.0_202404(2).pdf</x:v>
+        <x:v>Rizon4 用户手册_V3.0_zh-CN.pdf</x:v>
       </x:c>
       <x:c r="E18" s="15" t="str">
-        <x:v>sources/raw/02_非夕_Flexiv/02_Grav_星擎/星擎用户手册_V1.0_202404(2).pdf</x:v>
-      </x:c>
-      <x:c r="F18" s="15" t="str">
-        <x:v>2024-04</x:v>
-      </x:c>
+        <x:v>sources/raw/02_非夕_Flexiv/01_Rizon_拂晓/Rizon4 用户手册_V3.0_zh-CN.pdf</x:v>
+      </x:c>
+      <x:c r="F18" s="15" t="str"/>
       <x:c r="G18" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
@@ -5126,26 +5695,28 @@
         <x:v>中</x:v>
       </x:c>
       <x:c r="I18" s="15" t="str">
-        <x:v>末端执行器资料待结构化</x:v>
+        <x:v>待纳入机械臂专项对比</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="15" t="str">
-        <x:v>src_flexiv_ft_datasheet</x:v>
+        <x:v>src_flexiv_rizon_datasheet</x:v>
       </x:c>
       <x:c r="B19" s="15" t="str">
-        <x:v>flexiv_ft</x:v>
+        <x:v>flexiv_rizon</x:v>
       </x:c>
       <x:c r="C19" s="15" t="str">
         <x:v>供应商PDF</x:v>
       </x:c>
       <x:c r="D19" s="15" t="str">
-        <x:v>拂晓 F_T 传感器数据表_V1.0_zh-CN.pdf</x:v>
+        <x:v>拂晓(Rizon)机器人数据表_V2.0_202409.pdf</x:v>
       </x:c>
       <x:c r="E19" s="15" t="str">
-        <x:v>sources/raw/02_非夕_Flexiv/03_FT_拂晓传感器/拂晓 F_T 传感器数据表_V1.0_zh-CN.pdf</x:v>
-      </x:c>
-      <x:c r="F19" s="15" t="str"/>
+        <x:v>sources/raw/02_非夕_Flexiv/01_Rizon_拂晓/拂晓(Rizon)机器人数据表_V2.0_202409.pdf</x:v>
+      </x:c>
+      <x:c r="F19" s="15" t="str">
+        <x:v>2024-09</x:v>
+      </x:c>
       <x:c r="G19" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
@@ -5153,27 +5724,27 @@
         <x:v>中</x:v>
       </x:c>
       <x:c r="I19" s="15" t="str">
-        <x:v>力传感器资料待结构化</x:v>
+        <x:v>待纳入机械臂专项对比</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="15" t="str">
-        <x:v>src_tianji_marvin</x:v>
+        <x:v>src_flexiv_grav_manual</x:v>
       </x:c>
       <x:c r="B20" s="15" t="str">
-        <x:v>tianji_marvin_m6ccs</x:v>
+        <x:v>flexiv_grav</x:v>
       </x:c>
       <x:c r="C20" s="15" t="str">
         <x:v>供应商PDF</x:v>
       </x:c>
       <x:c r="D20" s="15" t="str">
-        <x:v>Marvin系列 三折页 250721-CN.pdf</x:v>
+        <x:v>星擎用户手册_V1.0_202404(2).pdf</x:v>
       </x:c>
       <x:c r="E20" s="15" t="str">
-        <x:v>sources/raw/03_天机智能_Marvin/01_Marvin双臂/Marvin系列 三折页 250721-CN.pdf</x:v>
+        <x:v>sources/raw/02_非夕_Flexiv/02_Grav_星擎/星擎用户手册_V1.0_202404(2).pdf</x:v>
       </x:c>
       <x:c r="F20" s="15" t="str">
-        <x:v>2025-07</x:v>
+        <x:v>2024-04</x:v>
       </x:c>
       <x:c r="G20" s="15" t="str">
         <x:v>2026-09-15</x:v>
@@ -5182,22 +5753,24 @@
         <x:v>中</x:v>
       </x:c>
       <x:c r="I20" s="15" t="str">
-        <x:v>单臂/双臂模块参数，不含标准底盘</x:v>
+        <x:v>末端执行器资料待结构化</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="15" t="str">
-        <x:v>src_material_index</x:v>
-      </x:c>
-      <x:c r="B21" s="15" t="str"/>
+        <x:v>src_flexiv_ft_datasheet</x:v>
+      </x:c>
+      <x:c r="B21" s="15" t="str">
+        <x:v>flexiv_ft</x:v>
+      </x:c>
       <x:c r="C21" s="15" t="str">
-        <x:v>内部索引</x:v>
+        <x:v>供应商PDF</x:v>
       </x:c>
       <x:c r="D21" s="15" t="str">
-        <x:v>供应链材料索引.md</x:v>
+        <x:v>拂晓 F_T 传感器数据表_V1.0_zh-CN.pdf</x:v>
       </x:c>
       <x:c r="E21" s="15" t="str">
-        <x:v>sources/raw/00_索引/供应链材料索引.md</x:v>
+        <x:v>sources/raw/02_非夕_Flexiv/03_FT_拂晓传感器/拂晓 F_T 传感器数据表_V1.0_zh-CN.pdf</x:v>
       </x:c>
       <x:c r="F21" s="15" t="str"/>
       <x:c r="G21" s="15" t="str">
@@ -5207,82 +5780,81 @@
         <x:v>中</x:v>
       </x:c>
       <x:c r="I21" s="15" t="str">
-        <x:v>原目录索引的归档副本</x:v>
+        <x:v>力传感器资料待结构化</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="15" t="str">
-        <x:v>src_boston_atlas</x:v>
+        <x:v>src_tianji_marvin</x:v>
       </x:c>
       <x:c r="B22" s="15" t="str">
-        <x:v>boston_atlas_2026</x:v>
+        <x:v>tianji_marvin_m6ccs</x:v>
       </x:c>
       <x:c r="C22" s="15" t="str">
-        <x:v>官方网站</x:v>
+        <x:v>供应商PDF</x:v>
       </x:c>
       <x:c r="D22" s="15" t="str">
-        <x:v>Atlas产品与规格</x:v>
+        <x:v>Marvin系列 三折页 250721-CN.pdf</x:v>
       </x:c>
       <x:c r="E22" s="15" t="str">
-        <x:v>https://bostondynamics.com/products/atlas/</x:v>
-      </x:c>
-      <x:c r="F22" s="15" t="str"/>
+        <x:v>sources/raw/03_天机智能_Marvin/01_Marvin双臂/Marvin系列 三折页 250721-CN.pdf</x:v>
+      </x:c>
+      <x:c r="F22" s="15" t="str">
+        <x:v>2025-07</x:v>
+      </x:c>
       <x:c r="G22" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
       <x:c r="H22" s="15" t="str">
-        <x:v>高</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="I22" s="15" t="str">
-        <x:v>披露56自由度、负载、续航、IP67、工作范围和Orbit集成</x:v>
+        <x:v>单臂/双臂模块参数，不含标准底盘</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="15" t="str">
-        <x:v>src_figure03_product</x:v>
-      </x:c>
-      <x:c r="B23" s="15" t="str">
-        <x:v>figure_03</x:v>
-      </x:c>
+        <x:v>src_material_index</x:v>
+      </x:c>
+      <x:c r="B23" s="15" t="str"/>
       <x:c r="C23" s="15" t="str">
-        <x:v>官方网站</x:v>
+        <x:v>内部索引</x:v>
       </x:c>
       <x:c r="D23" s="15" t="str">
-        <x:v>Figure 03产品页</x:v>
+        <x:v>供应链材料索引.md</x:v>
       </x:c>
       <x:c r="E23" s="15" t="str">
-        <x:v>https://www.figure.ai/figure</x:v>
+        <x:v>sources/raw/00_索引/供应链材料索引.md</x:v>
       </x:c>
       <x:c r="F23" s="15" t="str"/>
       <x:c r="G23" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
       <x:c r="H23" s="15" t="str">
-        <x:v>高</x:v>
+        <x:v>中</x:v>
       </x:c>
       <x:c r="I23" s="15" t="str">
-        <x:v>披露身高、重量、负载、速度和续航</x:v>
+        <x:v>原目录索引的归档副本</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
       <x:c r="A24" s="15" t="str">
-        <x:v>src_figure03_intro</x:v>
+        <x:v>src_boston_atlas</x:v>
       </x:c>
       <x:c r="B24" s="15" t="str">
-        <x:v>figure_03</x:v>
+        <x:v>boston_atlas_2026</x:v>
       </x:c>
       <x:c r="C24" s="15" t="str">
-        <x:v>官方技术文章</x:v>
+        <x:v>官方网站</x:v>
       </x:c>
       <x:c r="D24" s="15" t="str">
-        <x:v>Introducing Figure 03</x:v>
-      </x:c>
-      <x:c r="E24" s="15" t="str">
-        <x:v>https://www.figure.ai/news/introducing-figure-03</x:v>
-      </x:c>
-      <x:c r="F24" s="15" t="str">
-        <x:v>2025-10-09</x:v>
-      </x:c>
+        <x:v>Atlas产品与规格</x:v>
+      </x:c>
+      <x:c r="E24" s="15" t="e">
+        <x:f>HYPERLINK("https://bostondynamics.com/products/atlas/","https://bostondynamics.com/products/atlas/")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://bostondynamics.com/products/atlas/, friendlyName=https://bostondynamics.com/products/atlas/</x:v>
+      </x:c>
+      <x:c r="F24" s="15" t="str"/>
       <x:c r="G24" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
@@ -5290,28 +5862,27 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="I24" s="15" t="str">
-        <x:v>披露触觉、感知、充电、电池安全和量产设计</x:v>
+        <x:v>披露56自由度、负载、续航、IP67、工作范围和Orbit集成</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="15" t="str">
-        <x:v>src_figure03_bmw</x:v>
+        <x:v>src_figure03_product</x:v>
       </x:c>
       <x:c r="B25" s="15" t="str">
         <x:v>figure_03</x:v>
       </x:c>
       <x:c r="C25" s="15" t="str">
-        <x:v>官方客户进展</x:v>
+        <x:v>官方网站</x:v>
       </x:c>
       <x:c r="D25" s="15" t="str">
-        <x:v>F.03 Arrives at BMW</x:v>
-      </x:c>
-      <x:c r="E25" s="15" t="str">
-        <x:v>https://www.figure.ai/news/f-03-at-bmw</x:v>
-      </x:c>
-      <x:c r="F25" s="15" t="str">
-        <x:v>2026-06-30</x:v>
-      </x:c>
+        <x:v>Figure 03产品页</x:v>
+      </x:c>
+      <x:c r="E25" s="15" t="e">
+        <x:f>HYPERLINK("https://www.figure.ai/figure","https://www.figure.ai/figure")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://www.figure.ai/figure, friendlyName=https://www.figure.ai/figure</x:v>
+      </x:c>
+      <x:c r="F25" s="15" t="str"/>
       <x:c r="G25" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
@@ -5319,26 +5890,29 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="I25" s="15" t="str">
-        <x:v>披露BMW工厂物流验证和全身操作</x:v>
+        <x:v>披露身高、重量、负载、速度和续航</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="15" t="str">
-        <x:v>src_tesla_ai</x:v>
+        <x:v>src_figure03_intro</x:v>
       </x:c>
       <x:c r="B26" s="15" t="str">
-        <x:v>tesla_optimus</x:v>
+        <x:v>figure_03</x:v>
       </x:c>
       <x:c r="C26" s="15" t="str">
-        <x:v>官方网站</x:v>
+        <x:v>官方技术文章</x:v>
       </x:c>
       <x:c r="D26" s="15" t="str">
-        <x:v>Tesla AI and Robotics</x:v>
-      </x:c>
-      <x:c r="E26" s="15" t="str">
-        <x:v>https://www.tesla.com/AI</x:v>
-      </x:c>
-      <x:c r="F26" s="15" t="str"/>
+        <x:v>Introducing Figure 03</x:v>
+      </x:c>
+      <x:c r="E26" s="15" t="e">
+        <x:f>HYPERLINK("https://www.figure.ai/news/introducing-figure-03","https://www.figure.ai/news/introducing-figure-03")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://www.figure.ai/news/introducing-figure-03, friendlyName=https://www.figure.ai/news/introducing-figure-03</x:v>
+      </x:c>
+      <x:c r="F26" s="15" t="str">
+        <x:v>2025-10-09</x:v>
+      </x:c>
       <x:c r="G26" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
@@ -5346,27 +5920,28 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="I26" s="15" t="str">
-        <x:v>仅说明双足通用自主机器人目标；未给工程规格</x:v>
+        <x:v>披露触觉、感知、充电、电池安全和量产设计</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
       <x:c r="A27" s="15" t="str">
-        <x:v>src_tesla_2026q2</x:v>
+        <x:v>src_figure03_bmw</x:v>
       </x:c>
       <x:c r="B27" s="15" t="str">
-        <x:v>tesla_optimus</x:v>
+        <x:v>figure_03</x:v>
       </x:c>
       <x:c r="C27" s="15" t="str">
-        <x:v>官方投资者文件</x:v>
+        <x:v>官方客户进展</x:v>
       </x:c>
       <x:c r="D27" s="15" t="str">
-        <x:v>Tesla 2026 Q2 Update</x:v>
-      </x:c>
-      <x:c r="E27" s="15" t="str">
-        <x:v>https://ir.tesla.com/_flysystem/s3/sec/000162828026049213/tsla-20260722-gen.pdf</x:v>
+        <x:v>F.03 Arrives at BMW</x:v>
+      </x:c>
+      <x:c r="E27" s="15" t="e">
+        <x:f>HYPERLINK("https://www.figure.ai/news/f-03-at-bmw","https://www.figure.ai/news/f-03-at-bmw")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://www.figure.ai/news/f-03-at-bmw, friendlyName=https://www.figure.ai/news/f-03-at-bmw</x:v>
       </x:c>
       <x:c r="F27" s="15" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-06-30</x:v>
       </x:c>
       <x:c r="G27" s="15" t="str">
         <x:v>2026-09-15</x:v>
@@ -5375,24 +5950,25 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="I27" s="15" t="str">
-        <x:v>披露Optimus产线建设与训练数据用途；未给本体规格</x:v>
+        <x:v>披露BMW工厂物流验证和全身操作</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
       <x:c r="A28" s="15" t="str">
-        <x:v>src_limx_oli</x:v>
+        <x:v>src_tesla_ai</x:v>
       </x:c>
       <x:c r="B28" s="15" t="str">
-        <x:v>limx_oli_edu</x:v>
+        <x:v>tesla_optimus</x:v>
       </x:c>
       <x:c r="C28" s="15" t="str">
         <x:v>官方网站</x:v>
       </x:c>
       <x:c r="D28" s="15" t="str">
-        <x:v>LimX Oli产品参数</x:v>
-      </x:c>
-      <x:c r="E28" s="15" t="str">
-        <x:v>https://www.limxdynamics.com/zh/products/oli/spec</x:v>
+        <x:v>Tesla AI and Robotics</x:v>
+      </x:c>
+      <x:c r="E28" s="15" t="e">
+        <x:f>HYPERLINK("https://www.tesla.com/AI","https://www.tesla.com/AI")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://www.tesla.com/AI, friendlyName=https://www.tesla.com/AI</x:v>
       </x:c>
       <x:c r="F28" s="15" t="str"/>
       <x:c r="G28" s="15" t="str">
@@ -5402,26 +5978,29 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="I28" s="15" t="str">
-        <x:v>披露自由度、尺寸、负载、续航、算力和开发接口</x:v>
+        <x:v>仅说明双足通用自主机器人目标；未给工程规格</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="15" t="str">
-        <x:v>src_limx_tron2</x:v>
+        <x:v>src_tesla_2026q2</x:v>
       </x:c>
       <x:c r="B29" s="15" t="str">
-        <x:v>limx_tron2_dualarm</x:v>
+        <x:v>tesla_optimus</x:v>
       </x:c>
       <x:c r="C29" s="15" t="str">
-        <x:v>官方网站</x:v>
+        <x:v>官方投资者文件</x:v>
       </x:c>
       <x:c r="D29" s="15" t="str">
-        <x:v>TRON 2产品参数</x:v>
-      </x:c>
-      <x:c r="E29" s="15" t="str">
-        <x:v>https://www.limxdynamics.com/zh/products/tron2/spec</x:v>
-      </x:c>
-      <x:c r="F29" s="15" t="str"/>
+        <x:v>Tesla 2026 Q2 Update</x:v>
+      </x:c>
+      <x:c r="E29" s="15" t="e">
+        <x:f>HYPERLINK("https://ir.tesla.com/_flysystem/s3/sec/000162828026049213/tsla-20260722-gen.pdf","https://ir.tesla.com/_flysystem/s3/sec/000162828026049213/tsla-20260722-gen.pdf")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://ir.tesla.com/_flysystem/s3/sec/000162828026049213/tsla-20260722-gen.pdf, friendlyName=https://ir.tesla.com/_flysystem/s3/sec/000162828026049213/tsla-20260722-gen.pdf</x:v>
+      </x:c>
+      <x:c r="F29" s="15" t="str">
+        <x:v>2026-07-22</x:v>
+      </x:c>
       <x:c r="G29" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
@@ -5429,24 +6008,25 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="I29" s="15" t="str">
-        <x:v>披露双臂负载精度、多形态移动、接口和开发工具</x:v>
+        <x:v>披露Optimus产线建设与训练数据用途；未给本体规格</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="15" t="str">
-        <x:v>src_galaxea_r1pro_product</x:v>
+        <x:v>src_limx_oli</x:v>
       </x:c>
       <x:c r="B30" s="15" t="str">
-        <x:v>galaxea_r1pro_2026</x:v>
+        <x:v>limx_oli_edu</x:v>
       </x:c>
       <x:c r="C30" s="15" t="str">
         <x:v>官方网站</x:v>
       </x:c>
       <x:c r="D30" s="15" t="str">
-        <x:v>R1 Pro产品参数</x:v>
-      </x:c>
-      <x:c r="E30" s="15" t="str">
-        <x:v>https://galaxea-ai.com/cn/products/R1-Pro</x:v>
+        <x:v>LimX Oli产品参数</x:v>
+      </x:c>
+      <x:c r="E30" s="15" t="e">
+        <x:f>HYPERLINK("https://www.limxdynamics.com/zh/products/oli/spec","https://www.limxdynamics.com/zh/products/oli/spec")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://www.limxdynamics.com/zh/products/oli/spec, friendlyName=https://www.limxdynamics.com/zh/products/oli/spec</x:v>
       </x:c>
       <x:c r="F30" s="15" t="str"/>
       <x:c r="G30" s="15" t="str">
@@ -5456,24 +6036,25 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="I30" s="15" t="str">
-        <x:v>披露三舵轮全向底盘、双臂负载、工作空间和算力</x:v>
+        <x:v>披露自由度、尺寸、负载、续航、算力和开发接口</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
       <x:c r="A31" s="15" t="str">
-        <x:v>src_galaxea_r1pro_docs</x:v>
+        <x:v>src_limx_tron2</x:v>
       </x:c>
       <x:c r="B31" s="15" t="str">
-        <x:v>galaxea_r1pro_2026</x:v>
+        <x:v>limx_tron2_dualarm</x:v>
       </x:c>
       <x:c r="C31" s="15" t="str">
-        <x:v>官方开发文档</x:v>
+        <x:v>官方网站</x:v>
       </x:c>
       <x:c r="D31" s="15" t="str">
-        <x:v>R1 Pro 2026硬件说明</x:v>
-      </x:c>
-      <x:c r="E31" s="15" t="str">
-        <x:v>https://docs.galaxea-dynamics.com/R1Pro/docs/2026/</x:v>
+        <x:v>TRON 2产品参数</x:v>
+      </x:c>
+      <x:c r="E31" s="15" t="e">
+        <x:f>HYPERLINK("https://www.limxdynamics.com/zh/products/tron2/spec","https://www.limxdynamics.com/zh/products/tron2/spec")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://www.limxdynamics.com/zh/products/tron2/spec, friendlyName=https://www.limxdynamics.com/zh/products/tron2/spec</x:v>
       </x:c>
       <x:c r="F31" s="15" t="str"/>
       <x:c r="G31" s="15" t="str">
@@ -5483,28 +6064,27 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="I31" s="15" t="str">
-        <x:v>披露重量、电池、夹爪、接口和机械臂无制动器风险</x:v>
+        <x:v>披露双臂负载精度、多形态移动、接口和开发工具</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
       <x:c r="A32" s="15" t="str">
-        <x:v>src_tars_tianhai</x:v>
+        <x:v>src_galaxea_r1pro_product</x:v>
       </x:c>
       <x:c r="B32" s="15" t="str">
-        <x:v>tars_a1</x:v>
+        <x:v>galaxea_r1pro_2026</x:v>
       </x:c>
       <x:c r="C32" s="15" t="str">
-        <x:v>客户官方新闻</x:v>
+        <x:v>官方网站</x:v>
       </x:c>
       <x:c r="D32" s="15" t="str">
-        <x:v>天海电子与它石智航战略合作</x:v>
-      </x:c>
-      <x:c r="E32" s="15" t="str">
-        <x:v>https://www.thb.com.cn/content/details_17_319668.html</x:v>
-      </x:c>
-      <x:c r="F32" s="15" t="str">
-        <x:v>2026-06-28</x:v>
-      </x:c>
+        <x:v>R1 Pro产品参数</x:v>
+      </x:c>
+      <x:c r="E32" s="15" t="e">
+        <x:f>HYPERLINK("https://galaxea-ai.com/cn/products/R1-Pro","https://galaxea-ai.com/cn/products/R1-Pro")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://galaxea-ai.com/cn/products/R1-Pro, friendlyName=https://galaxea-ai.com/cn/products/R1-Pro</x:v>
+      </x:c>
+      <x:c r="F32" s="15" t="str"/>
       <x:c r="G32" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
@@ -5512,28 +6092,27 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="I32" s="15" t="str">
-        <x:v>确认汽车线束联合产线与近半年联合攻坚</x:v>
+        <x:v>披露三舵轮全向底盘、双臂负载、工作空间和算力</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="15" t="str">
-        <x:v>src_tars_shanghai</x:v>
+        <x:v>src_galaxea_r1pro_docs</x:v>
       </x:c>
       <x:c r="B33" s="15" t="str">
-        <x:v>tars_a1</x:v>
+        <x:v>galaxea_r1pro_2026</x:v>
       </x:c>
       <x:c r="C33" s="15" t="str">
-        <x:v>政府官方信息</x:v>
+        <x:v>官方开发文档</x:v>
       </x:c>
       <x:c r="D33" s="15" t="str">
-        <x:v>它石智航产业化闭环</x:v>
-      </x:c>
-      <x:c r="E33" s="15" t="str">
-        <x:v>https://www.sheitc.sh.gov.cn/zxxx/20260710/480d32461ca145e3bf067ce67dc6c203.html</x:v>
-      </x:c>
-      <x:c r="F33" s="15" t="str">
-        <x:v>2026-07-10</x:v>
-      </x:c>
+        <x:v>R1 Pro 2026硬件说明</x:v>
+      </x:c>
+      <x:c r="E33" s="15" t="e">
+        <x:f>HYPERLINK("https://docs.galaxea-dynamics.com/R1Pro/docs/2026/","https://docs.galaxea-dynamics.com/R1Pro/docs/2026/")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://docs.galaxea-dynamics.com/R1Pro/docs/2026/, friendlyName=https://docs.galaxea-dynamics.com/R1Pro/docs/2026/</x:v>
+      </x:c>
+      <x:c r="F33" s="15" t="str"/>
       <x:c r="G33" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
@@ -5541,26 +6120,29 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="I33" s="15" t="str">
-        <x:v>披露安波福百台计划、33类场景、46工位和DexHand</x:v>
+        <x:v>披露重量、电池、夹爪、接口和机械臂无制动器风险</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="15" t="str">
-        <x:v>src_tars_guinness</x:v>
+        <x:v>src_tars_tianhai</x:v>
       </x:c>
       <x:c r="B34" s="15" t="str">
         <x:v>tars_a1</x:v>
       </x:c>
       <x:c r="C34" s="15" t="str">
-        <x:v>独立纪录机构</x:v>
+        <x:v>客户官方新闻</x:v>
       </x:c>
       <x:c r="D34" s="15" t="str">
-        <x:v>Most sub-millimeter wire harness assembled by a robot in one hour</x:v>
-      </x:c>
-      <x:c r="E34" s="15" t="str">
-        <x:v>https://guinnessworldrecords.com.br/world-records/782788-most-sub-millimeter-wire-harness-assembled-by-a-robot-in-one-hour</x:v>
-      </x:c>
-      <x:c r="F34" s="15" t="str"/>
+        <x:v>天海电子与它石智航战略合作</x:v>
+      </x:c>
+      <x:c r="E34" s="15" t="e">
+        <x:f>HYPERLINK("https://www.thb.com.cn/content/details_17_319668.html","https://www.thb.com.cn/content/details_17_319668.html")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://www.thb.com.cn/content/details_17_319668.html, friendlyName=https://www.thb.com.cn/content/details_17_319668.html</x:v>
+      </x:c>
+      <x:c r="F34" s="15" t="str">
+        <x:v>2026-06-28</x:v>
+      </x:c>
       <x:c r="G34" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
@@ -5568,35 +6150,93 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="I34" s="15" t="str">
-        <x:v>确认一小时105次亚毫米线束装配纪录</x:v>
+        <x:v>确认汽车线束联合产线与近半年联合攻坚</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="15" t="str">
-        <x:v>src_tars_internal</x:v>
+        <x:v>src_tars_shanghai</x:v>
       </x:c>
       <x:c r="B35" s="15" t="str">
         <x:v>tars_a1</x:v>
       </x:c>
       <x:c r="C35" s="15" t="str">
-        <x:v>内部沟通</x:v>
+        <x:v>政府官方信息</x:v>
       </x:c>
       <x:c r="D35" s="15" t="str">
-        <x:v>它石线束部署与工程问题纪要</x:v>
-      </x:c>
-      <x:c r="E35" s="15" t="str">
-        <x:v>conversation-context:2026-09-15</x:v>
+        <x:v>它石智航产业化闭环</x:v>
+      </x:c>
+      <x:c r="E35" s="15" t="e">
+        <x:f>HYPERLINK("https://www.sheitc.sh.gov.cn/zxxx/20260710/480d32461ca145e3bf067ce67dc6c203.html","https://www.sheitc.sh.gov.cn/zxxx/20260710/480d32461ca145e3bf067ce67dc6c203.html")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://www.sheitc.sh.gov.cn/zxxx/20260710/480d32461ca145e3bf067ce67dc6c203.html, friendlyName=https://www.sheitc.sh.gov.cn/zxxx/20260710/480d32461ca145e3bf067ce67dc6c203.html</x:v>
       </x:c>
       <x:c r="F35" s="15" t="str">
-        <x:v>2026-09-15</x:v>
+        <x:v>2026-07-10</x:v>
       </x:c>
       <x:c r="G35" s="15" t="str">
         <x:v>2026-09-15</x:v>
       </x:c>
       <x:c r="H35" s="15" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="I35" s="15" t="str">
+        <x:v>披露安波福百台计划、33类场景、46工位和DexHand</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="42" customHeight="1">
+      <x:c r="A36" s="15" t="str">
+        <x:v>src_tars_guinness</x:v>
+      </x:c>
+      <x:c r="B36" s="15" t="str">
+        <x:v>tars_a1</x:v>
+      </x:c>
+      <x:c r="C36" s="15" t="str">
+        <x:v>独立纪录机构</x:v>
+      </x:c>
+      <x:c r="D36" s="15" t="str">
+        <x:v>Most sub-millimeter wire harness assembled by a robot in one hour</x:v>
+      </x:c>
+      <x:c r="E36" s="15" t="e">
+        <x:f>HYPERLINK("https://guinnessworldrecords.com.br/world-records/782788-most-sub-millimeter-wire-harness-assembled-by-a-robot-in-one-hour","https://guinnessworldrecords.com.br/world-records/782788-most-sub-millimeter-wire-harness-assembled-by-a-robot-in-one-hour")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://guinnessworldrecords.com.br/world-records/782788-most-sub-millimeter-wire-harness-assembled-by-a-robot-in-one-hour, friendlyName=https://guinnessworldrecords.com.br/world-records/782788-most-sub-millimeter-wire-harness-assembled-by-a-robot-in-one-hour</x:v>
+      </x:c>
+      <x:c r="F36" s="15" t="str"/>
+      <x:c r="G36" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H36" s="15" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="I36" s="15" t="str">
+        <x:v>确认一小时105次亚毫米线束装配纪录</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="42" customHeight="1">
+      <x:c r="A37" s="15" t="str">
+        <x:v>src_tars_internal</x:v>
+      </x:c>
+      <x:c r="B37" s="15" t="str">
+        <x:v>tars_a1</x:v>
+      </x:c>
+      <x:c r="C37" s="15" t="str">
+        <x:v>内部沟通</x:v>
+      </x:c>
+      <x:c r="D37" s="15" t="str">
+        <x:v>它石线束部署与工程问题纪要</x:v>
+      </x:c>
+      <x:c r="E37" s="15" t="str">
+        <x:v>conversation-context:2026-09-15</x:v>
+      </x:c>
+      <x:c r="F37" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="G37" s="15" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="H37" s="15" t="str">
         <x:v>待核验</x:v>
       </x:c>
-      <x:c r="I35" s="15" t="str">
+      <x:c r="I37" s="15" t="str">
         <x:v>反馈百台部署尚未达到要求并存在臂展、工装耗材、夹爪和MES依赖问题</x:v>
       </x:c>
     </x:row>
@@ -5606,7 +6246,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a5ac16dabe9421a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b3be9ef54844195"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>